<commit_message>
feat: numeração do calunga (número à esquerda/direita) e nome da fração
- migration 0018: perfis.numero_esq, numero_dir, nome_fracao; só o instrutor da turma altera (trigger 42501)
- mapa: números fora do quadro do símbolo; sem número, o nome de guerra continua ao lado
- nome da fração só no popup (colegas, próprio, situação, debriefing)
- painel do instrutor: editor de designação por aluno
- importação CSV/Edge Function e modelo Excel com as três colunas novas
- clientes toleram banco sem a 0018 (42703)

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ezu4AaNto4zS67SJhNsUXQ
</commit_message>
<xml_diff>
--- a/backend/seed/modelo-importacao-turma.xlsx
+++ b/backend/seed/modelo-importacao-turma.xlsx
@@ -231,7 +231,7 @@
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>OBRIGATÓRIO. É o que aparece no mapa ao lado do símbolo. Até 30 caracteres; mantenha curto.</t>
+        <t>OBRIGATÓRIO. Até 30 caracteres. Aparece ao lado do símbolo no mapa SÓ quando a pessoa não tem número à esquerda/direita (colunas numero_esq e numero_dir).</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
@@ -262,6 +262,21 @@
     <comment ref="J1" authorId="0" shapeId="0">
       <text>
         <t>Opcional. Vazio = símbolo genérico. Com valor: 6 ou 10 dígitos do catálogo. Coluna em formato Texto (não apaga zeros).</t>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0" shapeId="0">
+      <text>
+        <t>Opcional. Número À ESQUERDA do símbolo no mapa: a designação da fração (ex.: 1 para o 1º Pelotão). Até 4 caracteres. Vazio = sem número.</t>
+      </text>
+    </comment>
+    <comment ref="L1" authorId="0" shapeId="0">
+      <text>
+        <t>Opcional. Número À DIREITA do símbolo: a fração a que pertence (ex.: 2 para o 2º Esquadrão). Até 4 caracteres. Vazio = sem número.</t>
+      </text>
+    </comment>
+    <comment ref="M1" authorId="0" shapeId="0">
+      <text>
+        <t>Opcional. Nome curto da fração, texto livre, até 20 caracteres (ex.: 1º Pel / 2º Esqd). Aparece SÓ no popup do símbolo.</t>
       </text>
     </comment>
   </commentList>
@@ -557,7 +572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J301"/>
+  <dimension ref="A1:M301"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -570,6 +585,9 @@
     <col width="28" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -621,6 +639,21 @@
       <c r="J1" s="2" t="inlineStr">
         <is>
           <t>natureza_code</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>numero_esq</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>numero_dir</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>nome_fracao</t>
         </is>
       </c>
     </row>
@@ -635,6 +668,9 @@
       <c r="H2" s="3" t="n"/>
       <c r="I2" s="3" t="n"/>
       <c r="J2" s="3" t="n"/>
+      <c r="K2" s="3" t="n"/>
+      <c r="L2" s="3" t="n"/>
+      <c r="M2" s="3" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="n"/>
@@ -647,6 +683,9 @@
       <c r="H3" s="3" t="n"/>
       <c r="I3" s="3" t="n"/>
       <c r="J3" s="3" t="n"/>
+      <c r="K3" s="3" t="n"/>
+      <c r="L3" s="3" t="n"/>
+      <c r="M3" s="3" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n"/>
@@ -659,6 +698,9 @@
       <c r="H4" s="3" t="n"/>
       <c r="I4" s="3" t="n"/>
       <c r="J4" s="3" t="n"/>
+      <c r="K4" s="3" t="n"/>
+      <c r="L4" s="3" t="n"/>
+      <c r="M4" s="3" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n"/>
@@ -671,6 +713,9 @@
       <c r="H5" s="3" t="n"/>
       <c r="I5" s="3" t="n"/>
       <c r="J5" s="3" t="n"/>
+      <c r="K5" s="3" t="n"/>
+      <c r="L5" s="3" t="n"/>
+      <c r="M5" s="3" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n"/>
@@ -683,6 +728,9 @@
       <c r="H6" s="3" t="n"/>
       <c r="I6" s="3" t="n"/>
       <c r="J6" s="3" t="n"/>
+      <c r="K6" s="3" t="n"/>
+      <c r="L6" s="3" t="n"/>
+      <c r="M6" s="3" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n"/>
@@ -695,6 +743,9 @@
       <c r="H7" s="3" t="n"/>
       <c r="I7" s="3" t="n"/>
       <c r="J7" s="3" t="n"/>
+      <c r="K7" s="3" t="n"/>
+      <c r="L7" s="3" t="n"/>
+      <c r="M7" s="3" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n"/>
@@ -707,6 +758,9 @@
       <c r="H8" s="3" t="n"/>
       <c r="I8" s="3" t="n"/>
       <c r="J8" s="3" t="n"/>
+      <c r="K8" s="3" t="n"/>
+      <c r="L8" s="3" t="n"/>
+      <c r="M8" s="3" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n"/>
@@ -719,6 +773,9 @@
       <c r="H9" s="3" t="n"/>
       <c r="I9" s="3" t="n"/>
       <c r="J9" s="3" t="n"/>
+      <c r="K9" s="3" t="n"/>
+      <c r="L9" s="3" t="n"/>
+      <c r="M9" s="3" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n"/>
@@ -731,6 +788,9 @@
       <c r="H10" s="3" t="n"/>
       <c r="I10" s="3" t="n"/>
       <c r="J10" s="3" t="n"/>
+      <c r="K10" s="3" t="n"/>
+      <c r="L10" s="3" t="n"/>
+      <c r="M10" s="3" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n"/>
@@ -743,6 +803,9 @@
       <c r="H11" s="3" t="n"/>
       <c r="I11" s="3" t="n"/>
       <c r="J11" s="3" t="n"/>
+      <c r="K11" s="3" t="n"/>
+      <c r="L11" s="3" t="n"/>
+      <c r="M11" s="3" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n"/>
@@ -755,6 +818,9 @@
       <c r="H12" s="3" t="n"/>
       <c r="I12" s="3" t="n"/>
       <c r="J12" s="3" t="n"/>
+      <c r="K12" s="3" t="n"/>
+      <c r="L12" s="3" t="n"/>
+      <c r="M12" s="3" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n"/>
@@ -767,6 +833,9 @@
       <c r="H13" s="3" t="n"/>
       <c r="I13" s="3" t="n"/>
       <c r="J13" s="3" t="n"/>
+      <c r="K13" s="3" t="n"/>
+      <c r="L13" s="3" t="n"/>
+      <c r="M13" s="3" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n"/>
@@ -779,6 +848,9 @@
       <c r="H14" s="3" t="n"/>
       <c r="I14" s="3" t="n"/>
       <c r="J14" s="3" t="n"/>
+      <c r="K14" s="3" t="n"/>
+      <c r="L14" s="3" t="n"/>
+      <c r="M14" s="3" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="n"/>
@@ -791,6 +863,9 @@
       <c r="H15" s="3" t="n"/>
       <c r="I15" s="3" t="n"/>
       <c r="J15" s="3" t="n"/>
+      <c r="K15" s="3" t="n"/>
+      <c r="L15" s="3" t="n"/>
+      <c r="M15" s="3" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n"/>
@@ -803,6 +878,9 @@
       <c r="H16" s="3" t="n"/>
       <c r="I16" s="3" t="n"/>
       <c r="J16" s="3" t="n"/>
+      <c r="K16" s="3" t="n"/>
+      <c r="L16" s="3" t="n"/>
+      <c r="M16" s="3" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n"/>
@@ -815,6 +893,9 @@
       <c r="H17" s="3" t="n"/>
       <c r="I17" s="3" t="n"/>
       <c r="J17" s="3" t="n"/>
+      <c r="K17" s="3" t="n"/>
+      <c r="L17" s="3" t="n"/>
+      <c r="M17" s="3" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n"/>
@@ -827,6 +908,9 @@
       <c r="H18" s="3" t="n"/>
       <c r="I18" s="3" t="n"/>
       <c r="J18" s="3" t="n"/>
+      <c r="K18" s="3" t="n"/>
+      <c r="L18" s="3" t="n"/>
+      <c r="M18" s="3" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n"/>
@@ -839,6 +923,9 @@
       <c r="H19" s="3" t="n"/>
       <c r="I19" s="3" t="n"/>
       <c r="J19" s="3" t="n"/>
+      <c r="K19" s="3" t="n"/>
+      <c r="L19" s="3" t="n"/>
+      <c r="M19" s="3" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n"/>
@@ -851,6 +938,9 @@
       <c r="H20" s="3" t="n"/>
       <c r="I20" s="3" t="n"/>
       <c r="J20" s="3" t="n"/>
+      <c r="K20" s="3" t="n"/>
+      <c r="L20" s="3" t="n"/>
+      <c r="M20" s="3" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n"/>
@@ -863,6 +953,9 @@
       <c r="H21" s="3" t="n"/>
       <c r="I21" s="3" t="n"/>
       <c r="J21" s="3" t="n"/>
+      <c r="K21" s="3" t="n"/>
+      <c r="L21" s="3" t="n"/>
+      <c r="M21" s="3" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n"/>
@@ -875,6 +968,9 @@
       <c r="H22" s="3" t="n"/>
       <c r="I22" s="3" t="n"/>
       <c r="J22" s="3" t="n"/>
+      <c r="K22" s="3" t="n"/>
+      <c r="L22" s="3" t="n"/>
+      <c r="M22" s="3" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n"/>
@@ -887,6 +983,9 @@
       <c r="H23" s="3" t="n"/>
       <c r="I23" s="3" t="n"/>
       <c r="J23" s="3" t="n"/>
+      <c r="K23" s="3" t="n"/>
+      <c r="L23" s="3" t="n"/>
+      <c r="M23" s="3" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n"/>
@@ -899,6 +998,9 @@
       <c r="H24" s="3" t="n"/>
       <c r="I24" s="3" t="n"/>
       <c r="J24" s="3" t="n"/>
+      <c r="K24" s="3" t="n"/>
+      <c r="L24" s="3" t="n"/>
+      <c r="M24" s="3" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n"/>
@@ -911,6 +1013,9 @@
       <c r="H25" s="3" t="n"/>
       <c r="I25" s="3" t="n"/>
       <c r="J25" s="3" t="n"/>
+      <c r="K25" s="3" t="n"/>
+      <c r="L25" s="3" t="n"/>
+      <c r="M25" s="3" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n"/>
@@ -923,6 +1028,9 @@
       <c r="H26" s="3" t="n"/>
       <c r="I26" s="3" t="n"/>
       <c r="J26" s="3" t="n"/>
+      <c r="K26" s="3" t="n"/>
+      <c r="L26" s="3" t="n"/>
+      <c r="M26" s="3" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="n"/>
@@ -935,6 +1043,9 @@
       <c r="H27" s="3" t="n"/>
       <c r="I27" s="3" t="n"/>
       <c r="J27" s="3" t="n"/>
+      <c r="K27" s="3" t="n"/>
+      <c r="L27" s="3" t="n"/>
+      <c r="M27" s="3" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="n"/>
@@ -947,6 +1058,9 @@
       <c r="H28" s="3" t="n"/>
       <c r="I28" s="3" t="n"/>
       <c r="J28" s="3" t="n"/>
+      <c r="K28" s="3" t="n"/>
+      <c r="L28" s="3" t="n"/>
+      <c r="M28" s="3" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="3" t="n"/>
@@ -959,6 +1073,9 @@
       <c r="H29" s="3" t="n"/>
       <c r="I29" s="3" t="n"/>
       <c r="J29" s="3" t="n"/>
+      <c r="K29" s="3" t="n"/>
+      <c r="L29" s="3" t="n"/>
+      <c r="M29" s="3" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="n"/>
@@ -971,6 +1088,9 @@
       <c r="H30" s="3" t="n"/>
       <c r="I30" s="3" t="n"/>
       <c r="J30" s="3" t="n"/>
+      <c r="K30" s="3" t="n"/>
+      <c r="L30" s="3" t="n"/>
+      <c r="M30" s="3" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="3" t="n"/>
@@ -983,6 +1103,9 @@
       <c r="H31" s="3" t="n"/>
       <c r="I31" s="3" t="n"/>
       <c r="J31" s="3" t="n"/>
+      <c r="K31" s="3" t="n"/>
+      <c r="L31" s="3" t="n"/>
+      <c r="M31" s="3" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="3" t="n"/>
@@ -995,6 +1118,9 @@
       <c r="H32" s="3" t="n"/>
       <c r="I32" s="3" t="n"/>
       <c r="J32" s="3" t="n"/>
+      <c r="K32" s="3" t="n"/>
+      <c r="L32" s="3" t="n"/>
+      <c r="M32" s="3" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="3" t="n"/>
@@ -1007,6 +1133,9 @@
       <c r="H33" s="3" t="n"/>
       <c r="I33" s="3" t="n"/>
       <c r="J33" s="3" t="n"/>
+      <c r="K33" s="3" t="n"/>
+      <c r="L33" s="3" t="n"/>
+      <c r="M33" s="3" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="3" t="n"/>
@@ -1019,6 +1148,9 @@
       <c r="H34" s="3" t="n"/>
       <c r="I34" s="3" t="n"/>
       <c r="J34" s="3" t="n"/>
+      <c r="K34" s="3" t="n"/>
+      <c r="L34" s="3" t="n"/>
+      <c r="M34" s="3" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="3" t="n"/>
@@ -1031,6 +1163,9 @@
       <c r="H35" s="3" t="n"/>
       <c r="I35" s="3" t="n"/>
       <c r="J35" s="3" t="n"/>
+      <c r="K35" s="3" t="n"/>
+      <c r="L35" s="3" t="n"/>
+      <c r="M35" s="3" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="n"/>
@@ -1043,6 +1178,9 @@
       <c r="H36" s="3" t="n"/>
       <c r="I36" s="3" t="n"/>
       <c r="J36" s="3" t="n"/>
+      <c r="K36" s="3" t="n"/>
+      <c r="L36" s="3" t="n"/>
+      <c r="M36" s="3" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="3" t="n"/>
@@ -1055,6 +1193,9 @@
       <c r="H37" s="3" t="n"/>
       <c r="I37" s="3" t="n"/>
       <c r="J37" s="3" t="n"/>
+      <c r="K37" s="3" t="n"/>
+      <c r="L37" s="3" t="n"/>
+      <c r="M37" s="3" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="n"/>
@@ -1067,6 +1208,9 @@
       <c r="H38" s="3" t="n"/>
       <c r="I38" s="3" t="n"/>
       <c r="J38" s="3" t="n"/>
+      <c r="K38" s="3" t="n"/>
+      <c r="L38" s="3" t="n"/>
+      <c r="M38" s="3" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="3" t="n"/>
@@ -1079,6 +1223,9 @@
       <c r="H39" s="3" t="n"/>
       <c r="I39" s="3" t="n"/>
       <c r="J39" s="3" t="n"/>
+      <c r="K39" s="3" t="n"/>
+      <c r="L39" s="3" t="n"/>
+      <c r="M39" s="3" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="3" t="n"/>
@@ -1091,6 +1238,9 @@
       <c r="H40" s="3" t="n"/>
       <c r="I40" s="3" t="n"/>
       <c r="J40" s="3" t="n"/>
+      <c r="K40" s="3" t="n"/>
+      <c r="L40" s="3" t="n"/>
+      <c r="M40" s="3" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="3" t="n"/>
@@ -1103,6 +1253,9 @@
       <c r="H41" s="3" t="n"/>
       <c r="I41" s="3" t="n"/>
       <c r="J41" s="3" t="n"/>
+      <c r="K41" s="3" t="n"/>
+      <c r="L41" s="3" t="n"/>
+      <c r="M41" s="3" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="3" t="n"/>
@@ -1115,6 +1268,9 @@
       <c r="H42" s="3" t="n"/>
       <c r="I42" s="3" t="n"/>
       <c r="J42" s="3" t="n"/>
+      <c r="K42" s="3" t="n"/>
+      <c r="L42" s="3" t="n"/>
+      <c r="M42" s="3" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="3" t="n"/>
@@ -1127,6 +1283,9 @@
       <c r="H43" s="3" t="n"/>
       <c r="I43" s="3" t="n"/>
       <c r="J43" s="3" t="n"/>
+      <c r="K43" s="3" t="n"/>
+      <c r="L43" s="3" t="n"/>
+      <c r="M43" s="3" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="3" t="n"/>
@@ -1139,6 +1298,9 @@
       <c r="H44" s="3" t="n"/>
       <c r="I44" s="3" t="n"/>
       <c r="J44" s="3" t="n"/>
+      <c r="K44" s="3" t="n"/>
+      <c r="L44" s="3" t="n"/>
+      <c r="M44" s="3" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="3" t="n"/>
@@ -1151,6 +1313,9 @@
       <c r="H45" s="3" t="n"/>
       <c r="I45" s="3" t="n"/>
       <c r="J45" s="3" t="n"/>
+      <c r="K45" s="3" t="n"/>
+      <c r="L45" s="3" t="n"/>
+      <c r="M45" s="3" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="3" t="n"/>
@@ -1163,6 +1328,9 @@
       <c r="H46" s="3" t="n"/>
       <c r="I46" s="3" t="n"/>
       <c r="J46" s="3" t="n"/>
+      <c r="K46" s="3" t="n"/>
+      <c r="L46" s="3" t="n"/>
+      <c r="M46" s="3" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="3" t="n"/>
@@ -1175,6 +1343,9 @@
       <c r="H47" s="3" t="n"/>
       <c r="I47" s="3" t="n"/>
       <c r="J47" s="3" t="n"/>
+      <c r="K47" s="3" t="n"/>
+      <c r="L47" s="3" t="n"/>
+      <c r="M47" s="3" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="3" t="n"/>
@@ -1187,6 +1358,9 @@
       <c r="H48" s="3" t="n"/>
       <c r="I48" s="3" t="n"/>
       <c r="J48" s="3" t="n"/>
+      <c r="K48" s="3" t="n"/>
+      <c r="L48" s="3" t="n"/>
+      <c r="M48" s="3" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="3" t="n"/>
@@ -1199,6 +1373,9 @@
       <c r="H49" s="3" t="n"/>
       <c r="I49" s="3" t="n"/>
       <c r="J49" s="3" t="n"/>
+      <c r="K49" s="3" t="n"/>
+      <c r="L49" s="3" t="n"/>
+      <c r="M49" s="3" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="3" t="n"/>
@@ -1211,6 +1388,9 @@
       <c r="H50" s="3" t="n"/>
       <c r="I50" s="3" t="n"/>
       <c r="J50" s="3" t="n"/>
+      <c r="K50" s="3" t="n"/>
+      <c r="L50" s="3" t="n"/>
+      <c r="M50" s="3" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="3" t="n"/>
@@ -1223,6 +1403,9 @@
       <c r="H51" s="3" t="n"/>
       <c r="I51" s="3" t="n"/>
       <c r="J51" s="3" t="n"/>
+      <c r="K51" s="3" t="n"/>
+      <c r="L51" s="3" t="n"/>
+      <c r="M51" s="3" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="3" t="n"/>
@@ -1235,6 +1418,9 @@
       <c r="H52" s="3" t="n"/>
       <c r="I52" s="3" t="n"/>
       <c r="J52" s="3" t="n"/>
+      <c r="K52" s="3" t="n"/>
+      <c r="L52" s="3" t="n"/>
+      <c r="M52" s="3" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="3" t="n"/>
@@ -1247,6 +1433,9 @@
       <c r="H53" s="3" t="n"/>
       <c r="I53" s="3" t="n"/>
       <c r="J53" s="3" t="n"/>
+      <c r="K53" s="3" t="n"/>
+      <c r="L53" s="3" t="n"/>
+      <c r="M53" s="3" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="3" t="n"/>
@@ -1259,6 +1448,9 @@
       <c r="H54" s="3" t="n"/>
       <c r="I54" s="3" t="n"/>
       <c r="J54" s="3" t="n"/>
+      <c r="K54" s="3" t="n"/>
+      <c r="L54" s="3" t="n"/>
+      <c r="M54" s="3" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="3" t="n"/>
@@ -1271,6 +1463,9 @@
       <c r="H55" s="3" t="n"/>
       <c r="I55" s="3" t="n"/>
       <c r="J55" s="3" t="n"/>
+      <c r="K55" s="3" t="n"/>
+      <c r="L55" s="3" t="n"/>
+      <c r="M55" s="3" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="3" t="n"/>
@@ -1283,6 +1478,9 @@
       <c r="H56" s="3" t="n"/>
       <c r="I56" s="3" t="n"/>
       <c r="J56" s="3" t="n"/>
+      <c r="K56" s="3" t="n"/>
+      <c r="L56" s="3" t="n"/>
+      <c r="M56" s="3" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="3" t="n"/>
@@ -1295,6 +1493,9 @@
       <c r="H57" s="3" t="n"/>
       <c r="I57" s="3" t="n"/>
       <c r="J57" s="3" t="n"/>
+      <c r="K57" s="3" t="n"/>
+      <c r="L57" s="3" t="n"/>
+      <c r="M57" s="3" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="3" t="n"/>
@@ -1307,6 +1508,9 @@
       <c r="H58" s="3" t="n"/>
       <c r="I58" s="3" t="n"/>
       <c r="J58" s="3" t="n"/>
+      <c r="K58" s="3" t="n"/>
+      <c r="L58" s="3" t="n"/>
+      <c r="M58" s="3" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="3" t="n"/>
@@ -1319,6 +1523,9 @@
       <c r="H59" s="3" t="n"/>
       <c r="I59" s="3" t="n"/>
       <c r="J59" s="3" t="n"/>
+      <c r="K59" s="3" t="n"/>
+      <c r="L59" s="3" t="n"/>
+      <c r="M59" s="3" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="3" t="n"/>
@@ -1331,6 +1538,9 @@
       <c r="H60" s="3" t="n"/>
       <c r="I60" s="3" t="n"/>
       <c r="J60" s="3" t="n"/>
+      <c r="K60" s="3" t="n"/>
+      <c r="L60" s="3" t="n"/>
+      <c r="M60" s="3" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="3" t="n"/>
@@ -1343,6 +1553,9 @@
       <c r="H61" s="3" t="n"/>
       <c r="I61" s="3" t="n"/>
       <c r="J61" s="3" t="n"/>
+      <c r="K61" s="3" t="n"/>
+      <c r="L61" s="3" t="n"/>
+      <c r="M61" s="3" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="3" t="n"/>
@@ -1355,6 +1568,9 @@
       <c r="H62" s="3" t="n"/>
       <c r="I62" s="3" t="n"/>
       <c r="J62" s="3" t="n"/>
+      <c r="K62" s="3" t="n"/>
+      <c r="L62" s="3" t="n"/>
+      <c r="M62" s="3" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="3" t="n"/>
@@ -1367,6 +1583,9 @@
       <c r="H63" s="3" t="n"/>
       <c r="I63" s="3" t="n"/>
       <c r="J63" s="3" t="n"/>
+      <c r="K63" s="3" t="n"/>
+      <c r="L63" s="3" t="n"/>
+      <c r="M63" s="3" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="3" t="n"/>
@@ -1379,6 +1598,9 @@
       <c r="H64" s="3" t="n"/>
       <c r="I64" s="3" t="n"/>
       <c r="J64" s="3" t="n"/>
+      <c r="K64" s="3" t="n"/>
+      <c r="L64" s="3" t="n"/>
+      <c r="M64" s="3" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="3" t="n"/>
@@ -1391,6 +1613,9 @@
       <c r="H65" s="3" t="n"/>
       <c r="I65" s="3" t="n"/>
       <c r="J65" s="3" t="n"/>
+      <c r="K65" s="3" t="n"/>
+      <c r="L65" s="3" t="n"/>
+      <c r="M65" s="3" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="3" t="n"/>
@@ -1403,6 +1628,9 @@
       <c r="H66" s="3" t="n"/>
       <c r="I66" s="3" t="n"/>
       <c r="J66" s="3" t="n"/>
+      <c r="K66" s="3" t="n"/>
+      <c r="L66" s="3" t="n"/>
+      <c r="M66" s="3" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="3" t="n"/>
@@ -1415,6 +1643,9 @@
       <c r="H67" s="3" t="n"/>
       <c r="I67" s="3" t="n"/>
       <c r="J67" s="3" t="n"/>
+      <c r="K67" s="3" t="n"/>
+      <c r="L67" s="3" t="n"/>
+      <c r="M67" s="3" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="3" t="n"/>
@@ -1427,6 +1658,9 @@
       <c r="H68" s="3" t="n"/>
       <c r="I68" s="3" t="n"/>
       <c r="J68" s="3" t="n"/>
+      <c r="K68" s="3" t="n"/>
+      <c r="L68" s="3" t="n"/>
+      <c r="M68" s="3" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="3" t="n"/>
@@ -1439,6 +1673,9 @@
       <c r="H69" s="3" t="n"/>
       <c r="I69" s="3" t="n"/>
       <c r="J69" s="3" t="n"/>
+      <c r="K69" s="3" t="n"/>
+      <c r="L69" s="3" t="n"/>
+      <c r="M69" s="3" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="3" t="n"/>
@@ -1451,6 +1688,9 @@
       <c r="H70" s="3" t="n"/>
       <c r="I70" s="3" t="n"/>
       <c r="J70" s="3" t="n"/>
+      <c r="K70" s="3" t="n"/>
+      <c r="L70" s="3" t="n"/>
+      <c r="M70" s="3" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="3" t="n"/>
@@ -1463,6 +1703,9 @@
       <c r="H71" s="3" t="n"/>
       <c r="I71" s="3" t="n"/>
       <c r="J71" s="3" t="n"/>
+      <c r="K71" s="3" t="n"/>
+      <c r="L71" s="3" t="n"/>
+      <c r="M71" s="3" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="3" t="n"/>
@@ -1475,6 +1718,9 @@
       <c r="H72" s="3" t="n"/>
       <c r="I72" s="3" t="n"/>
       <c r="J72" s="3" t="n"/>
+      <c r="K72" s="3" t="n"/>
+      <c r="L72" s="3" t="n"/>
+      <c r="M72" s="3" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="3" t="n"/>
@@ -1487,6 +1733,9 @@
       <c r="H73" s="3" t="n"/>
       <c r="I73" s="3" t="n"/>
       <c r="J73" s="3" t="n"/>
+      <c r="K73" s="3" t="n"/>
+      <c r="L73" s="3" t="n"/>
+      <c r="M73" s="3" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="3" t="n"/>
@@ -1499,6 +1748,9 @@
       <c r="H74" s="3" t="n"/>
       <c r="I74" s="3" t="n"/>
       <c r="J74" s="3" t="n"/>
+      <c r="K74" s="3" t="n"/>
+      <c r="L74" s="3" t="n"/>
+      <c r="M74" s="3" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="3" t="n"/>
@@ -1511,6 +1763,9 @@
       <c r="H75" s="3" t="n"/>
       <c r="I75" s="3" t="n"/>
       <c r="J75" s="3" t="n"/>
+      <c r="K75" s="3" t="n"/>
+      <c r="L75" s="3" t="n"/>
+      <c r="M75" s="3" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="3" t="n"/>
@@ -1523,6 +1778,9 @@
       <c r="H76" s="3" t="n"/>
       <c r="I76" s="3" t="n"/>
       <c r="J76" s="3" t="n"/>
+      <c r="K76" s="3" t="n"/>
+      <c r="L76" s="3" t="n"/>
+      <c r="M76" s="3" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="3" t="n"/>
@@ -1535,6 +1793,9 @@
       <c r="H77" s="3" t="n"/>
       <c r="I77" s="3" t="n"/>
       <c r="J77" s="3" t="n"/>
+      <c r="K77" s="3" t="n"/>
+      <c r="L77" s="3" t="n"/>
+      <c r="M77" s="3" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="3" t="n"/>
@@ -1547,6 +1808,9 @@
       <c r="H78" s="3" t="n"/>
       <c r="I78" s="3" t="n"/>
       <c r="J78" s="3" t="n"/>
+      <c r="K78" s="3" t="n"/>
+      <c r="L78" s="3" t="n"/>
+      <c r="M78" s="3" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="3" t="n"/>
@@ -1559,6 +1823,9 @@
       <c r="H79" s="3" t="n"/>
       <c r="I79" s="3" t="n"/>
       <c r="J79" s="3" t="n"/>
+      <c r="K79" s="3" t="n"/>
+      <c r="L79" s="3" t="n"/>
+      <c r="M79" s="3" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="3" t="n"/>
@@ -1571,6 +1838,9 @@
       <c r="H80" s="3" t="n"/>
       <c r="I80" s="3" t="n"/>
       <c r="J80" s="3" t="n"/>
+      <c r="K80" s="3" t="n"/>
+      <c r="L80" s="3" t="n"/>
+      <c r="M80" s="3" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="3" t="n"/>
@@ -1583,6 +1853,9 @@
       <c r="H81" s="3" t="n"/>
       <c r="I81" s="3" t="n"/>
       <c r="J81" s="3" t="n"/>
+      <c r="K81" s="3" t="n"/>
+      <c r="L81" s="3" t="n"/>
+      <c r="M81" s="3" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="3" t="n"/>
@@ -1595,6 +1868,9 @@
       <c r="H82" s="3" t="n"/>
       <c r="I82" s="3" t="n"/>
       <c r="J82" s="3" t="n"/>
+      <c r="K82" s="3" t="n"/>
+      <c r="L82" s="3" t="n"/>
+      <c r="M82" s="3" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="3" t="n"/>
@@ -1607,6 +1883,9 @@
       <c r="H83" s="3" t="n"/>
       <c r="I83" s="3" t="n"/>
       <c r="J83" s="3" t="n"/>
+      <c r="K83" s="3" t="n"/>
+      <c r="L83" s="3" t="n"/>
+      <c r="M83" s="3" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="3" t="n"/>
@@ -1619,6 +1898,9 @@
       <c r="H84" s="3" t="n"/>
       <c r="I84" s="3" t="n"/>
       <c r="J84" s="3" t="n"/>
+      <c r="K84" s="3" t="n"/>
+      <c r="L84" s="3" t="n"/>
+      <c r="M84" s="3" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="3" t="n"/>
@@ -1631,6 +1913,9 @@
       <c r="H85" s="3" t="n"/>
       <c r="I85" s="3" t="n"/>
       <c r="J85" s="3" t="n"/>
+      <c r="K85" s="3" t="n"/>
+      <c r="L85" s="3" t="n"/>
+      <c r="M85" s="3" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="3" t="n"/>
@@ -1643,6 +1928,9 @@
       <c r="H86" s="3" t="n"/>
       <c r="I86" s="3" t="n"/>
       <c r="J86" s="3" t="n"/>
+      <c r="K86" s="3" t="n"/>
+      <c r="L86" s="3" t="n"/>
+      <c r="M86" s="3" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="3" t="n"/>
@@ -1655,6 +1943,9 @@
       <c r="H87" s="3" t="n"/>
       <c r="I87" s="3" t="n"/>
       <c r="J87" s="3" t="n"/>
+      <c r="K87" s="3" t="n"/>
+      <c r="L87" s="3" t="n"/>
+      <c r="M87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="3" t="n"/>
@@ -1667,6 +1958,9 @@
       <c r="H88" s="3" t="n"/>
       <c r="I88" s="3" t="n"/>
       <c r="J88" s="3" t="n"/>
+      <c r="K88" s="3" t="n"/>
+      <c r="L88" s="3" t="n"/>
+      <c r="M88" s="3" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="3" t="n"/>
@@ -1679,6 +1973,9 @@
       <c r="H89" s="3" t="n"/>
       <c r="I89" s="3" t="n"/>
       <c r="J89" s="3" t="n"/>
+      <c r="K89" s="3" t="n"/>
+      <c r="L89" s="3" t="n"/>
+      <c r="M89" s="3" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="3" t="n"/>
@@ -1691,6 +1988,9 @@
       <c r="H90" s="3" t="n"/>
       <c r="I90" s="3" t="n"/>
       <c r="J90" s="3" t="n"/>
+      <c r="K90" s="3" t="n"/>
+      <c r="L90" s="3" t="n"/>
+      <c r="M90" s="3" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="3" t="n"/>
@@ -1703,6 +2003,9 @@
       <c r="H91" s="3" t="n"/>
       <c r="I91" s="3" t="n"/>
       <c r="J91" s="3" t="n"/>
+      <c r="K91" s="3" t="n"/>
+      <c r="L91" s="3" t="n"/>
+      <c r="M91" s="3" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="3" t="n"/>
@@ -1715,6 +2018,9 @@
       <c r="H92" s="3" t="n"/>
       <c r="I92" s="3" t="n"/>
       <c r="J92" s="3" t="n"/>
+      <c r="K92" s="3" t="n"/>
+      <c r="L92" s="3" t="n"/>
+      <c r="M92" s="3" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="3" t="n"/>
@@ -1727,6 +2033,9 @@
       <c r="H93" s="3" t="n"/>
       <c r="I93" s="3" t="n"/>
       <c r="J93" s="3" t="n"/>
+      <c r="K93" s="3" t="n"/>
+      <c r="L93" s="3" t="n"/>
+      <c r="M93" s="3" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="3" t="n"/>
@@ -1739,6 +2048,9 @@
       <c r="H94" s="3" t="n"/>
       <c r="I94" s="3" t="n"/>
       <c r="J94" s="3" t="n"/>
+      <c r="K94" s="3" t="n"/>
+      <c r="L94" s="3" t="n"/>
+      <c r="M94" s="3" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="3" t="n"/>
@@ -1751,6 +2063,9 @@
       <c r="H95" s="3" t="n"/>
       <c r="I95" s="3" t="n"/>
       <c r="J95" s="3" t="n"/>
+      <c r="K95" s="3" t="n"/>
+      <c r="L95" s="3" t="n"/>
+      <c r="M95" s="3" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="3" t="n"/>
@@ -1763,6 +2078,9 @@
       <c r="H96" s="3" t="n"/>
       <c r="I96" s="3" t="n"/>
       <c r="J96" s="3" t="n"/>
+      <c r="K96" s="3" t="n"/>
+      <c r="L96" s="3" t="n"/>
+      <c r="M96" s="3" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="3" t="n"/>
@@ -1775,6 +2093,9 @@
       <c r="H97" s="3" t="n"/>
       <c r="I97" s="3" t="n"/>
       <c r="J97" s="3" t="n"/>
+      <c r="K97" s="3" t="n"/>
+      <c r="L97" s="3" t="n"/>
+      <c r="M97" s="3" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="3" t="n"/>
@@ -1787,6 +2108,9 @@
       <c r="H98" s="3" t="n"/>
       <c r="I98" s="3" t="n"/>
       <c r="J98" s="3" t="n"/>
+      <c r="K98" s="3" t="n"/>
+      <c r="L98" s="3" t="n"/>
+      <c r="M98" s="3" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="3" t="n"/>
@@ -1799,6 +2123,9 @@
       <c r="H99" s="3" t="n"/>
       <c r="I99" s="3" t="n"/>
       <c r="J99" s="3" t="n"/>
+      <c r="K99" s="3" t="n"/>
+      <c r="L99" s="3" t="n"/>
+      <c r="M99" s="3" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="3" t="n"/>
@@ -1811,6 +2138,9 @@
       <c r="H100" s="3" t="n"/>
       <c r="I100" s="3" t="n"/>
       <c r="J100" s="3" t="n"/>
+      <c r="K100" s="3" t="n"/>
+      <c r="L100" s="3" t="n"/>
+      <c r="M100" s="3" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="3" t="n"/>
@@ -1823,6 +2153,9 @@
       <c r="H101" s="3" t="n"/>
       <c r="I101" s="3" t="n"/>
       <c r="J101" s="3" t="n"/>
+      <c r="K101" s="3" t="n"/>
+      <c r="L101" s="3" t="n"/>
+      <c r="M101" s="3" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="3" t="n"/>
@@ -1835,6 +2168,9 @@
       <c r="H102" s="3" t="n"/>
       <c r="I102" s="3" t="n"/>
       <c r="J102" s="3" t="n"/>
+      <c r="K102" s="3" t="n"/>
+      <c r="L102" s="3" t="n"/>
+      <c r="M102" s="3" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="3" t="n"/>
@@ -1847,6 +2183,9 @@
       <c r="H103" s="3" t="n"/>
       <c r="I103" s="3" t="n"/>
       <c r="J103" s="3" t="n"/>
+      <c r="K103" s="3" t="n"/>
+      <c r="L103" s="3" t="n"/>
+      <c r="M103" s="3" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="3" t="n"/>
@@ -1859,6 +2198,9 @@
       <c r="H104" s="3" t="n"/>
       <c r="I104" s="3" t="n"/>
       <c r="J104" s="3" t="n"/>
+      <c r="K104" s="3" t="n"/>
+      <c r="L104" s="3" t="n"/>
+      <c r="M104" s="3" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="3" t="n"/>
@@ -1871,6 +2213,9 @@
       <c r="H105" s="3" t="n"/>
       <c r="I105" s="3" t="n"/>
       <c r="J105" s="3" t="n"/>
+      <c r="K105" s="3" t="n"/>
+      <c r="L105" s="3" t="n"/>
+      <c r="M105" s="3" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="3" t="n"/>
@@ -1883,6 +2228,9 @@
       <c r="H106" s="3" t="n"/>
       <c r="I106" s="3" t="n"/>
       <c r="J106" s="3" t="n"/>
+      <c r="K106" s="3" t="n"/>
+      <c r="L106" s="3" t="n"/>
+      <c r="M106" s="3" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="3" t="n"/>
@@ -1895,6 +2243,9 @@
       <c r="H107" s="3" t="n"/>
       <c r="I107" s="3" t="n"/>
       <c r="J107" s="3" t="n"/>
+      <c r="K107" s="3" t="n"/>
+      <c r="L107" s="3" t="n"/>
+      <c r="M107" s="3" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="3" t="n"/>
@@ -1907,6 +2258,9 @@
       <c r="H108" s="3" t="n"/>
       <c r="I108" s="3" t="n"/>
       <c r="J108" s="3" t="n"/>
+      <c r="K108" s="3" t="n"/>
+      <c r="L108" s="3" t="n"/>
+      <c r="M108" s="3" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="3" t="n"/>
@@ -1919,6 +2273,9 @@
       <c r="H109" s="3" t="n"/>
       <c r="I109" s="3" t="n"/>
       <c r="J109" s="3" t="n"/>
+      <c r="K109" s="3" t="n"/>
+      <c r="L109" s="3" t="n"/>
+      <c r="M109" s="3" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="3" t="n"/>
@@ -1931,6 +2288,9 @@
       <c r="H110" s="3" t="n"/>
       <c r="I110" s="3" t="n"/>
       <c r="J110" s="3" t="n"/>
+      <c r="K110" s="3" t="n"/>
+      <c r="L110" s="3" t="n"/>
+      <c r="M110" s="3" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="3" t="n"/>
@@ -1943,6 +2303,9 @@
       <c r="H111" s="3" t="n"/>
       <c r="I111" s="3" t="n"/>
       <c r="J111" s="3" t="n"/>
+      <c r="K111" s="3" t="n"/>
+      <c r="L111" s="3" t="n"/>
+      <c r="M111" s="3" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="3" t="n"/>
@@ -1955,6 +2318,9 @@
       <c r="H112" s="3" t="n"/>
       <c r="I112" s="3" t="n"/>
       <c r="J112" s="3" t="n"/>
+      <c r="K112" s="3" t="n"/>
+      <c r="L112" s="3" t="n"/>
+      <c r="M112" s="3" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="3" t="n"/>
@@ -1967,6 +2333,9 @@
       <c r="H113" s="3" t="n"/>
       <c r="I113" s="3" t="n"/>
       <c r="J113" s="3" t="n"/>
+      <c r="K113" s="3" t="n"/>
+      <c r="L113" s="3" t="n"/>
+      <c r="M113" s="3" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="3" t="n"/>
@@ -1979,6 +2348,9 @@
       <c r="H114" s="3" t="n"/>
       <c r="I114" s="3" t="n"/>
       <c r="J114" s="3" t="n"/>
+      <c r="K114" s="3" t="n"/>
+      <c r="L114" s="3" t="n"/>
+      <c r="M114" s="3" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="3" t="n"/>
@@ -1991,6 +2363,9 @@
       <c r="H115" s="3" t="n"/>
       <c r="I115" s="3" t="n"/>
       <c r="J115" s="3" t="n"/>
+      <c r="K115" s="3" t="n"/>
+      <c r="L115" s="3" t="n"/>
+      <c r="M115" s="3" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="3" t="n"/>
@@ -2003,6 +2378,9 @@
       <c r="H116" s="3" t="n"/>
       <c r="I116" s="3" t="n"/>
       <c r="J116" s="3" t="n"/>
+      <c r="K116" s="3" t="n"/>
+      <c r="L116" s="3" t="n"/>
+      <c r="M116" s="3" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="3" t="n"/>
@@ -2015,6 +2393,9 @@
       <c r="H117" s="3" t="n"/>
       <c r="I117" s="3" t="n"/>
       <c r="J117" s="3" t="n"/>
+      <c r="K117" s="3" t="n"/>
+      <c r="L117" s="3" t="n"/>
+      <c r="M117" s="3" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="3" t="n"/>
@@ -2027,6 +2408,9 @@
       <c r="H118" s="3" t="n"/>
       <c r="I118" s="3" t="n"/>
       <c r="J118" s="3" t="n"/>
+      <c r="K118" s="3" t="n"/>
+      <c r="L118" s="3" t="n"/>
+      <c r="M118" s="3" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="3" t="n"/>
@@ -2039,6 +2423,9 @@
       <c r="H119" s="3" t="n"/>
       <c r="I119" s="3" t="n"/>
       <c r="J119" s="3" t="n"/>
+      <c r="K119" s="3" t="n"/>
+      <c r="L119" s="3" t="n"/>
+      <c r="M119" s="3" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="3" t="n"/>
@@ -2051,6 +2438,9 @@
       <c r="H120" s="3" t="n"/>
       <c r="I120" s="3" t="n"/>
       <c r="J120" s="3" t="n"/>
+      <c r="K120" s="3" t="n"/>
+      <c r="L120" s="3" t="n"/>
+      <c r="M120" s="3" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="3" t="n"/>
@@ -2063,6 +2453,9 @@
       <c r="H121" s="3" t="n"/>
       <c r="I121" s="3" t="n"/>
       <c r="J121" s="3" t="n"/>
+      <c r="K121" s="3" t="n"/>
+      <c r="L121" s="3" t="n"/>
+      <c r="M121" s="3" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="3" t="n"/>
@@ -2075,6 +2468,9 @@
       <c r="H122" s="3" t="n"/>
       <c r="I122" s="3" t="n"/>
       <c r="J122" s="3" t="n"/>
+      <c r="K122" s="3" t="n"/>
+      <c r="L122" s="3" t="n"/>
+      <c r="M122" s="3" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="3" t="n"/>
@@ -2087,6 +2483,9 @@
       <c r="H123" s="3" t="n"/>
       <c r="I123" s="3" t="n"/>
       <c r="J123" s="3" t="n"/>
+      <c r="K123" s="3" t="n"/>
+      <c r="L123" s="3" t="n"/>
+      <c r="M123" s="3" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="3" t="n"/>
@@ -2099,6 +2498,9 @@
       <c r="H124" s="3" t="n"/>
       <c r="I124" s="3" t="n"/>
       <c r="J124" s="3" t="n"/>
+      <c r="K124" s="3" t="n"/>
+      <c r="L124" s="3" t="n"/>
+      <c r="M124" s="3" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="3" t="n"/>
@@ -2111,6 +2513,9 @@
       <c r="H125" s="3" t="n"/>
       <c r="I125" s="3" t="n"/>
       <c r="J125" s="3" t="n"/>
+      <c r="K125" s="3" t="n"/>
+      <c r="L125" s="3" t="n"/>
+      <c r="M125" s="3" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="3" t="n"/>
@@ -2123,6 +2528,9 @@
       <c r="H126" s="3" t="n"/>
       <c r="I126" s="3" t="n"/>
       <c r="J126" s="3" t="n"/>
+      <c r="K126" s="3" t="n"/>
+      <c r="L126" s="3" t="n"/>
+      <c r="M126" s="3" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="3" t="n"/>
@@ -2135,6 +2543,9 @@
       <c r="H127" s="3" t="n"/>
       <c r="I127" s="3" t="n"/>
       <c r="J127" s="3" t="n"/>
+      <c r="K127" s="3" t="n"/>
+      <c r="L127" s="3" t="n"/>
+      <c r="M127" s="3" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="3" t="n"/>
@@ -2147,6 +2558,9 @@
       <c r="H128" s="3" t="n"/>
       <c r="I128" s="3" t="n"/>
       <c r="J128" s="3" t="n"/>
+      <c r="K128" s="3" t="n"/>
+      <c r="L128" s="3" t="n"/>
+      <c r="M128" s="3" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="3" t="n"/>
@@ -2159,6 +2573,9 @@
       <c r="H129" s="3" t="n"/>
       <c r="I129" s="3" t="n"/>
       <c r="J129" s="3" t="n"/>
+      <c r="K129" s="3" t="n"/>
+      <c r="L129" s="3" t="n"/>
+      <c r="M129" s="3" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="3" t="n"/>
@@ -2171,6 +2588,9 @@
       <c r="H130" s="3" t="n"/>
       <c r="I130" s="3" t="n"/>
       <c r="J130" s="3" t="n"/>
+      <c r="K130" s="3" t="n"/>
+      <c r="L130" s="3" t="n"/>
+      <c r="M130" s="3" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="3" t="n"/>
@@ -2183,6 +2603,9 @@
       <c r="H131" s="3" t="n"/>
       <c r="I131" s="3" t="n"/>
       <c r="J131" s="3" t="n"/>
+      <c r="K131" s="3" t="n"/>
+      <c r="L131" s="3" t="n"/>
+      <c r="M131" s="3" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="3" t="n"/>
@@ -2195,6 +2618,9 @@
       <c r="H132" s="3" t="n"/>
       <c r="I132" s="3" t="n"/>
       <c r="J132" s="3" t="n"/>
+      <c r="K132" s="3" t="n"/>
+      <c r="L132" s="3" t="n"/>
+      <c r="M132" s="3" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="3" t="n"/>
@@ -2207,6 +2633,9 @@
       <c r="H133" s="3" t="n"/>
       <c r="I133" s="3" t="n"/>
       <c r="J133" s="3" t="n"/>
+      <c r="K133" s="3" t="n"/>
+      <c r="L133" s="3" t="n"/>
+      <c r="M133" s="3" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="3" t="n"/>
@@ -2219,6 +2648,9 @@
       <c r="H134" s="3" t="n"/>
       <c r="I134" s="3" t="n"/>
       <c r="J134" s="3" t="n"/>
+      <c r="K134" s="3" t="n"/>
+      <c r="L134" s="3" t="n"/>
+      <c r="M134" s="3" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="3" t="n"/>
@@ -2231,6 +2663,9 @@
       <c r="H135" s="3" t="n"/>
       <c r="I135" s="3" t="n"/>
       <c r="J135" s="3" t="n"/>
+      <c r="K135" s="3" t="n"/>
+      <c r="L135" s="3" t="n"/>
+      <c r="M135" s="3" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="3" t="n"/>
@@ -2243,6 +2678,9 @@
       <c r="H136" s="3" t="n"/>
       <c r="I136" s="3" t="n"/>
       <c r="J136" s="3" t="n"/>
+      <c r="K136" s="3" t="n"/>
+      <c r="L136" s="3" t="n"/>
+      <c r="M136" s="3" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="3" t="n"/>
@@ -2255,6 +2693,9 @@
       <c r="H137" s="3" t="n"/>
       <c r="I137" s="3" t="n"/>
       <c r="J137" s="3" t="n"/>
+      <c r="K137" s="3" t="n"/>
+      <c r="L137" s="3" t="n"/>
+      <c r="M137" s="3" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="3" t="n"/>
@@ -2267,6 +2708,9 @@
       <c r="H138" s="3" t="n"/>
       <c r="I138" s="3" t="n"/>
       <c r="J138" s="3" t="n"/>
+      <c r="K138" s="3" t="n"/>
+      <c r="L138" s="3" t="n"/>
+      <c r="M138" s="3" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="3" t="n"/>
@@ -2279,6 +2723,9 @@
       <c r="H139" s="3" t="n"/>
       <c r="I139" s="3" t="n"/>
       <c r="J139" s="3" t="n"/>
+      <c r="K139" s="3" t="n"/>
+      <c r="L139" s="3" t="n"/>
+      <c r="M139" s="3" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="3" t="n"/>
@@ -2291,6 +2738,9 @@
       <c r="H140" s="3" t="n"/>
       <c r="I140" s="3" t="n"/>
       <c r="J140" s="3" t="n"/>
+      <c r="K140" s="3" t="n"/>
+      <c r="L140" s="3" t="n"/>
+      <c r="M140" s="3" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="3" t="n"/>
@@ -2303,6 +2753,9 @@
       <c r="H141" s="3" t="n"/>
       <c r="I141" s="3" t="n"/>
       <c r="J141" s="3" t="n"/>
+      <c r="K141" s="3" t="n"/>
+      <c r="L141" s="3" t="n"/>
+      <c r="M141" s="3" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="3" t="n"/>
@@ -2315,6 +2768,9 @@
       <c r="H142" s="3" t="n"/>
       <c r="I142" s="3" t="n"/>
       <c r="J142" s="3" t="n"/>
+      <c r="K142" s="3" t="n"/>
+      <c r="L142" s="3" t="n"/>
+      <c r="M142" s="3" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="3" t="n"/>
@@ -2327,6 +2783,9 @@
       <c r="H143" s="3" t="n"/>
       <c r="I143" s="3" t="n"/>
       <c r="J143" s="3" t="n"/>
+      <c r="K143" s="3" t="n"/>
+      <c r="L143" s="3" t="n"/>
+      <c r="M143" s="3" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="3" t="n"/>
@@ -2339,6 +2798,9 @@
       <c r="H144" s="3" t="n"/>
       <c r="I144" s="3" t="n"/>
       <c r="J144" s="3" t="n"/>
+      <c r="K144" s="3" t="n"/>
+      <c r="L144" s="3" t="n"/>
+      <c r="M144" s="3" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="3" t="n"/>
@@ -2351,6 +2813,9 @@
       <c r="H145" s="3" t="n"/>
       <c r="I145" s="3" t="n"/>
       <c r="J145" s="3" t="n"/>
+      <c r="K145" s="3" t="n"/>
+      <c r="L145" s="3" t="n"/>
+      <c r="M145" s="3" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="3" t="n"/>
@@ -2363,6 +2828,9 @@
       <c r="H146" s="3" t="n"/>
       <c r="I146" s="3" t="n"/>
       <c r="J146" s="3" t="n"/>
+      <c r="K146" s="3" t="n"/>
+      <c r="L146" s="3" t="n"/>
+      <c r="M146" s="3" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="3" t="n"/>
@@ -2375,6 +2843,9 @@
       <c r="H147" s="3" t="n"/>
       <c r="I147" s="3" t="n"/>
       <c r="J147" s="3" t="n"/>
+      <c r="K147" s="3" t="n"/>
+      <c r="L147" s="3" t="n"/>
+      <c r="M147" s="3" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="3" t="n"/>
@@ -2387,6 +2858,9 @@
       <c r="H148" s="3" t="n"/>
       <c r="I148" s="3" t="n"/>
       <c r="J148" s="3" t="n"/>
+      <c r="K148" s="3" t="n"/>
+      <c r="L148" s="3" t="n"/>
+      <c r="M148" s="3" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="3" t="n"/>
@@ -2399,6 +2873,9 @@
       <c r="H149" s="3" t="n"/>
       <c r="I149" s="3" t="n"/>
       <c r="J149" s="3" t="n"/>
+      <c r="K149" s="3" t="n"/>
+      <c r="L149" s="3" t="n"/>
+      <c r="M149" s="3" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="3" t="n"/>
@@ -2411,6 +2888,9 @@
       <c r="H150" s="3" t="n"/>
       <c r="I150" s="3" t="n"/>
       <c r="J150" s="3" t="n"/>
+      <c r="K150" s="3" t="n"/>
+      <c r="L150" s="3" t="n"/>
+      <c r="M150" s="3" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="3" t="n"/>
@@ -2423,6 +2903,9 @@
       <c r="H151" s="3" t="n"/>
       <c r="I151" s="3" t="n"/>
       <c r="J151" s="3" t="n"/>
+      <c r="K151" s="3" t="n"/>
+      <c r="L151" s="3" t="n"/>
+      <c r="M151" s="3" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="3" t="n"/>
@@ -2435,6 +2918,9 @@
       <c r="H152" s="3" t="n"/>
       <c r="I152" s="3" t="n"/>
       <c r="J152" s="3" t="n"/>
+      <c r="K152" s="3" t="n"/>
+      <c r="L152" s="3" t="n"/>
+      <c r="M152" s="3" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="3" t="n"/>
@@ -2447,6 +2933,9 @@
       <c r="H153" s="3" t="n"/>
       <c r="I153" s="3" t="n"/>
       <c r="J153" s="3" t="n"/>
+      <c r="K153" s="3" t="n"/>
+      <c r="L153" s="3" t="n"/>
+      <c r="M153" s="3" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="3" t="n"/>
@@ -2459,6 +2948,9 @@
       <c r="H154" s="3" t="n"/>
       <c r="I154" s="3" t="n"/>
       <c r="J154" s="3" t="n"/>
+      <c r="K154" s="3" t="n"/>
+      <c r="L154" s="3" t="n"/>
+      <c r="M154" s="3" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="3" t="n"/>
@@ -2471,6 +2963,9 @@
       <c r="H155" s="3" t="n"/>
       <c r="I155" s="3" t="n"/>
       <c r="J155" s="3" t="n"/>
+      <c r="K155" s="3" t="n"/>
+      <c r="L155" s="3" t="n"/>
+      <c r="M155" s="3" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="3" t="n"/>
@@ -2483,6 +2978,9 @@
       <c r="H156" s="3" t="n"/>
       <c r="I156" s="3" t="n"/>
       <c r="J156" s="3" t="n"/>
+      <c r="K156" s="3" t="n"/>
+      <c r="L156" s="3" t="n"/>
+      <c r="M156" s="3" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="3" t="n"/>
@@ -2495,6 +2993,9 @@
       <c r="H157" s="3" t="n"/>
       <c r="I157" s="3" t="n"/>
       <c r="J157" s="3" t="n"/>
+      <c r="K157" s="3" t="n"/>
+      <c r="L157" s="3" t="n"/>
+      <c r="M157" s="3" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="3" t="n"/>
@@ -2507,6 +3008,9 @@
       <c r="H158" s="3" t="n"/>
       <c r="I158" s="3" t="n"/>
       <c r="J158" s="3" t="n"/>
+      <c r="K158" s="3" t="n"/>
+      <c r="L158" s="3" t="n"/>
+      <c r="M158" s="3" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="3" t="n"/>
@@ -2519,6 +3023,9 @@
       <c r="H159" s="3" t="n"/>
       <c r="I159" s="3" t="n"/>
       <c r="J159" s="3" t="n"/>
+      <c r="K159" s="3" t="n"/>
+      <c r="L159" s="3" t="n"/>
+      <c r="M159" s="3" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="3" t="n"/>
@@ -2531,6 +3038,9 @@
       <c r="H160" s="3" t="n"/>
       <c r="I160" s="3" t="n"/>
       <c r="J160" s="3" t="n"/>
+      <c r="K160" s="3" t="n"/>
+      <c r="L160" s="3" t="n"/>
+      <c r="M160" s="3" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="3" t="n"/>
@@ -2543,6 +3053,9 @@
       <c r="H161" s="3" t="n"/>
       <c r="I161" s="3" t="n"/>
       <c r="J161" s="3" t="n"/>
+      <c r="K161" s="3" t="n"/>
+      <c r="L161" s="3" t="n"/>
+      <c r="M161" s="3" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="3" t="n"/>
@@ -2555,6 +3068,9 @@
       <c r="H162" s="3" t="n"/>
       <c r="I162" s="3" t="n"/>
       <c r="J162" s="3" t="n"/>
+      <c r="K162" s="3" t="n"/>
+      <c r="L162" s="3" t="n"/>
+      <c r="M162" s="3" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="3" t="n"/>
@@ -2567,6 +3083,9 @@
       <c r="H163" s="3" t="n"/>
       <c r="I163" s="3" t="n"/>
       <c r="J163" s="3" t="n"/>
+      <c r="K163" s="3" t="n"/>
+      <c r="L163" s="3" t="n"/>
+      <c r="M163" s="3" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="3" t="n"/>
@@ -2579,6 +3098,9 @@
       <c r="H164" s="3" t="n"/>
       <c r="I164" s="3" t="n"/>
       <c r="J164" s="3" t="n"/>
+      <c r="K164" s="3" t="n"/>
+      <c r="L164" s="3" t="n"/>
+      <c r="M164" s="3" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="3" t="n"/>
@@ -2591,6 +3113,9 @@
       <c r="H165" s="3" t="n"/>
       <c r="I165" s="3" t="n"/>
       <c r="J165" s="3" t="n"/>
+      <c r="K165" s="3" t="n"/>
+      <c r="L165" s="3" t="n"/>
+      <c r="M165" s="3" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="3" t="n"/>
@@ -2603,6 +3128,9 @@
       <c r="H166" s="3" t="n"/>
       <c r="I166" s="3" t="n"/>
       <c r="J166" s="3" t="n"/>
+      <c r="K166" s="3" t="n"/>
+      <c r="L166" s="3" t="n"/>
+      <c r="M166" s="3" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="3" t="n"/>
@@ -2615,6 +3143,9 @@
       <c r="H167" s="3" t="n"/>
       <c r="I167" s="3" t="n"/>
       <c r="J167" s="3" t="n"/>
+      <c r="K167" s="3" t="n"/>
+      <c r="L167" s="3" t="n"/>
+      <c r="M167" s="3" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="3" t="n"/>
@@ -2627,6 +3158,9 @@
       <c r="H168" s="3" t="n"/>
       <c r="I168" s="3" t="n"/>
       <c r="J168" s="3" t="n"/>
+      <c r="K168" s="3" t="n"/>
+      <c r="L168" s="3" t="n"/>
+      <c r="M168" s="3" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="3" t="n"/>
@@ -2639,6 +3173,9 @@
       <c r="H169" s="3" t="n"/>
       <c r="I169" s="3" t="n"/>
       <c r="J169" s="3" t="n"/>
+      <c r="K169" s="3" t="n"/>
+      <c r="L169" s="3" t="n"/>
+      <c r="M169" s="3" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="3" t="n"/>
@@ -2651,6 +3188,9 @@
       <c r="H170" s="3" t="n"/>
       <c r="I170" s="3" t="n"/>
       <c r="J170" s="3" t="n"/>
+      <c r="K170" s="3" t="n"/>
+      <c r="L170" s="3" t="n"/>
+      <c r="M170" s="3" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="3" t="n"/>
@@ -2663,6 +3203,9 @@
       <c r="H171" s="3" t="n"/>
       <c r="I171" s="3" t="n"/>
       <c r="J171" s="3" t="n"/>
+      <c r="K171" s="3" t="n"/>
+      <c r="L171" s="3" t="n"/>
+      <c r="M171" s="3" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="3" t="n"/>
@@ -2675,6 +3218,9 @@
       <c r="H172" s="3" t="n"/>
       <c r="I172" s="3" t="n"/>
       <c r="J172" s="3" t="n"/>
+      <c r="K172" s="3" t="n"/>
+      <c r="L172" s="3" t="n"/>
+      <c r="M172" s="3" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="3" t="n"/>
@@ -2687,6 +3233,9 @@
       <c r="H173" s="3" t="n"/>
       <c r="I173" s="3" t="n"/>
       <c r="J173" s="3" t="n"/>
+      <c r="K173" s="3" t="n"/>
+      <c r="L173" s="3" t="n"/>
+      <c r="M173" s="3" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="3" t="n"/>
@@ -2699,6 +3248,9 @@
       <c r="H174" s="3" t="n"/>
       <c r="I174" s="3" t="n"/>
       <c r="J174" s="3" t="n"/>
+      <c r="K174" s="3" t="n"/>
+      <c r="L174" s="3" t="n"/>
+      <c r="M174" s="3" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="3" t="n"/>
@@ -2711,6 +3263,9 @@
       <c r="H175" s="3" t="n"/>
       <c r="I175" s="3" t="n"/>
       <c r="J175" s="3" t="n"/>
+      <c r="K175" s="3" t="n"/>
+      <c r="L175" s="3" t="n"/>
+      <c r="M175" s="3" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="3" t="n"/>
@@ -2723,6 +3278,9 @@
       <c r="H176" s="3" t="n"/>
       <c r="I176" s="3" t="n"/>
       <c r="J176" s="3" t="n"/>
+      <c r="K176" s="3" t="n"/>
+      <c r="L176" s="3" t="n"/>
+      <c r="M176" s="3" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="3" t="n"/>
@@ -2735,6 +3293,9 @@
       <c r="H177" s="3" t="n"/>
       <c r="I177" s="3" t="n"/>
       <c r="J177" s="3" t="n"/>
+      <c r="K177" s="3" t="n"/>
+      <c r="L177" s="3" t="n"/>
+      <c r="M177" s="3" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="3" t="n"/>
@@ -2747,6 +3308,9 @@
       <c r="H178" s="3" t="n"/>
       <c r="I178" s="3" t="n"/>
       <c r="J178" s="3" t="n"/>
+      <c r="K178" s="3" t="n"/>
+      <c r="L178" s="3" t="n"/>
+      <c r="M178" s="3" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="3" t="n"/>
@@ -2759,6 +3323,9 @@
       <c r="H179" s="3" t="n"/>
       <c r="I179" s="3" t="n"/>
       <c r="J179" s="3" t="n"/>
+      <c r="K179" s="3" t="n"/>
+      <c r="L179" s="3" t="n"/>
+      <c r="M179" s="3" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="3" t="n"/>
@@ -2771,6 +3338,9 @@
       <c r="H180" s="3" t="n"/>
       <c r="I180" s="3" t="n"/>
       <c r="J180" s="3" t="n"/>
+      <c r="K180" s="3" t="n"/>
+      <c r="L180" s="3" t="n"/>
+      <c r="M180" s="3" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="3" t="n"/>
@@ -2783,6 +3353,9 @@
       <c r="H181" s="3" t="n"/>
       <c r="I181" s="3" t="n"/>
       <c r="J181" s="3" t="n"/>
+      <c r="K181" s="3" t="n"/>
+      <c r="L181" s="3" t="n"/>
+      <c r="M181" s="3" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="3" t="n"/>
@@ -2795,6 +3368,9 @@
       <c r="H182" s="3" t="n"/>
       <c r="I182" s="3" t="n"/>
       <c r="J182" s="3" t="n"/>
+      <c r="K182" s="3" t="n"/>
+      <c r="L182" s="3" t="n"/>
+      <c r="M182" s="3" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="3" t="n"/>
@@ -2807,6 +3383,9 @@
       <c r="H183" s="3" t="n"/>
       <c r="I183" s="3" t="n"/>
       <c r="J183" s="3" t="n"/>
+      <c r="K183" s="3" t="n"/>
+      <c r="L183" s="3" t="n"/>
+      <c r="M183" s="3" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="3" t="n"/>
@@ -2819,6 +3398,9 @@
       <c r="H184" s="3" t="n"/>
       <c r="I184" s="3" t="n"/>
       <c r="J184" s="3" t="n"/>
+      <c r="K184" s="3" t="n"/>
+      <c r="L184" s="3" t="n"/>
+      <c r="M184" s="3" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="3" t="n"/>
@@ -2831,6 +3413,9 @@
       <c r="H185" s="3" t="n"/>
       <c r="I185" s="3" t="n"/>
       <c r="J185" s="3" t="n"/>
+      <c r="K185" s="3" t="n"/>
+      <c r="L185" s="3" t="n"/>
+      <c r="M185" s="3" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="3" t="n"/>
@@ -2843,6 +3428,9 @@
       <c r="H186" s="3" t="n"/>
       <c r="I186" s="3" t="n"/>
       <c r="J186" s="3" t="n"/>
+      <c r="K186" s="3" t="n"/>
+      <c r="L186" s="3" t="n"/>
+      <c r="M186" s="3" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="3" t="n"/>
@@ -2855,6 +3443,9 @@
       <c r="H187" s="3" t="n"/>
       <c r="I187" s="3" t="n"/>
       <c r="J187" s="3" t="n"/>
+      <c r="K187" s="3" t="n"/>
+      <c r="L187" s="3" t="n"/>
+      <c r="M187" s="3" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="3" t="n"/>
@@ -2867,6 +3458,9 @@
       <c r="H188" s="3" t="n"/>
       <c r="I188" s="3" t="n"/>
       <c r="J188" s="3" t="n"/>
+      <c r="K188" s="3" t="n"/>
+      <c r="L188" s="3" t="n"/>
+      <c r="M188" s="3" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="3" t="n"/>
@@ -2879,6 +3473,9 @@
       <c r="H189" s="3" t="n"/>
       <c r="I189" s="3" t="n"/>
       <c r="J189" s="3" t="n"/>
+      <c r="K189" s="3" t="n"/>
+      <c r="L189" s="3" t="n"/>
+      <c r="M189" s="3" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="3" t="n"/>
@@ -2891,6 +3488,9 @@
       <c r="H190" s="3" t="n"/>
       <c r="I190" s="3" t="n"/>
       <c r="J190" s="3" t="n"/>
+      <c r="K190" s="3" t="n"/>
+      <c r="L190" s="3" t="n"/>
+      <c r="M190" s="3" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="3" t="n"/>
@@ -2903,6 +3503,9 @@
       <c r="H191" s="3" t="n"/>
       <c r="I191" s="3" t="n"/>
       <c r="J191" s="3" t="n"/>
+      <c r="K191" s="3" t="n"/>
+      <c r="L191" s="3" t="n"/>
+      <c r="M191" s="3" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="3" t="n"/>
@@ -2915,6 +3518,9 @@
       <c r="H192" s="3" t="n"/>
       <c r="I192" s="3" t="n"/>
       <c r="J192" s="3" t="n"/>
+      <c r="K192" s="3" t="n"/>
+      <c r="L192" s="3" t="n"/>
+      <c r="M192" s="3" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="3" t="n"/>
@@ -2927,6 +3533,9 @@
       <c r="H193" s="3" t="n"/>
       <c r="I193" s="3" t="n"/>
       <c r="J193" s="3" t="n"/>
+      <c r="K193" s="3" t="n"/>
+      <c r="L193" s="3" t="n"/>
+      <c r="M193" s="3" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="3" t="n"/>
@@ -2939,6 +3548,9 @@
       <c r="H194" s="3" t="n"/>
       <c r="I194" s="3" t="n"/>
       <c r="J194" s="3" t="n"/>
+      <c r="K194" s="3" t="n"/>
+      <c r="L194" s="3" t="n"/>
+      <c r="M194" s="3" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="3" t="n"/>
@@ -2951,6 +3563,9 @@
       <c r="H195" s="3" t="n"/>
       <c r="I195" s="3" t="n"/>
       <c r="J195" s="3" t="n"/>
+      <c r="K195" s="3" t="n"/>
+      <c r="L195" s="3" t="n"/>
+      <c r="M195" s="3" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="3" t="n"/>
@@ -2963,6 +3578,9 @@
       <c r="H196" s="3" t="n"/>
       <c r="I196" s="3" t="n"/>
       <c r="J196" s="3" t="n"/>
+      <c r="K196" s="3" t="n"/>
+      <c r="L196" s="3" t="n"/>
+      <c r="M196" s="3" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="3" t="n"/>
@@ -2975,6 +3593,9 @@
       <c r="H197" s="3" t="n"/>
       <c r="I197" s="3" t="n"/>
       <c r="J197" s="3" t="n"/>
+      <c r="K197" s="3" t="n"/>
+      <c r="L197" s="3" t="n"/>
+      <c r="M197" s="3" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="3" t="n"/>
@@ -2987,6 +3608,9 @@
       <c r="H198" s="3" t="n"/>
       <c r="I198" s="3" t="n"/>
       <c r="J198" s="3" t="n"/>
+      <c r="K198" s="3" t="n"/>
+      <c r="L198" s="3" t="n"/>
+      <c r="M198" s="3" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="3" t="n"/>
@@ -2999,6 +3623,9 @@
       <c r="H199" s="3" t="n"/>
       <c r="I199" s="3" t="n"/>
       <c r="J199" s="3" t="n"/>
+      <c r="K199" s="3" t="n"/>
+      <c r="L199" s="3" t="n"/>
+      <c r="M199" s="3" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="3" t="n"/>
@@ -3011,6 +3638,9 @@
       <c r="H200" s="3" t="n"/>
       <c r="I200" s="3" t="n"/>
       <c r="J200" s="3" t="n"/>
+      <c r="K200" s="3" t="n"/>
+      <c r="L200" s="3" t="n"/>
+      <c r="M200" s="3" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="3" t="n"/>
@@ -3023,6 +3653,9 @@
       <c r="H201" s="3" t="n"/>
       <c r="I201" s="3" t="n"/>
       <c r="J201" s="3" t="n"/>
+      <c r="K201" s="3" t="n"/>
+      <c r="L201" s="3" t="n"/>
+      <c r="M201" s="3" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="3" t="n"/>
@@ -3035,6 +3668,9 @@
       <c r="H202" s="3" t="n"/>
       <c r="I202" s="3" t="n"/>
       <c r="J202" s="3" t="n"/>
+      <c r="K202" s="3" t="n"/>
+      <c r="L202" s="3" t="n"/>
+      <c r="M202" s="3" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="3" t="n"/>
@@ -3047,6 +3683,9 @@
       <c r="H203" s="3" t="n"/>
       <c r="I203" s="3" t="n"/>
       <c r="J203" s="3" t="n"/>
+      <c r="K203" s="3" t="n"/>
+      <c r="L203" s="3" t="n"/>
+      <c r="M203" s="3" t="n"/>
     </row>
     <row r="204">
       <c r="A204" s="3" t="n"/>
@@ -3059,6 +3698,9 @@
       <c r="H204" s="3" t="n"/>
       <c r="I204" s="3" t="n"/>
       <c r="J204" s="3" t="n"/>
+      <c r="K204" s="3" t="n"/>
+      <c r="L204" s="3" t="n"/>
+      <c r="M204" s="3" t="n"/>
     </row>
     <row r="205">
       <c r="A205" s="3" t="n"/>
@@ -3071,6 +3713,9 @@
       <c r="H205" s="3" t="n"/>
       <c r="I205" s="3" t="n"/>
       <c r="J205" s="3" t="n"/>
+      <c r="K205" s="3" t="n"/>
+      <c r="L205" s="3" t="n"/>
+      <c r="M205" s="3" t="n"/>
     </row>
     <row r="206">
       <c r="A206" s="3" t="n"/>
@@ -3083,6 +3728,9 @@
       <c r="H206" s="3" t="n"/>
       <c r="I206" s="3" t="n"/>
       <c r="J206" s="3" t="n"/>
+      <c r="K206" s="3" t="n"/>
+      <c r="L206" s="3" t="n"/>
+      <c r="M206" s="3" t="n"/>
     </row>
     <row r="207">
       <c r="A207" s="3" t="n"/>
@@ -3095,6 +3743,9 @@
       <c r="H207" s="3" t="n"/>
       <c r="I207" s="3" t="n"/>
       <c r="J207" s="3" t="n"/>
+      <c r="K207" s="3" t="n"/>
+      <c r="L207" s="3" t="n"/>
+      <c r="M207" s="3" t="n"/>
     </row>
     <row r="208">
       <c r="A208" s="3" t="n"/>
@@ -3107,6 +3758,9 @@
       <c r="H208" s="3" t="n"/>
       <c r="I208" s="3" t="n"/>
       <c r="J208" s="3" t="n"/>
+      <c r="K208" s="3" t="n"/>
+      <c r="L208" s="3" t="n"/>
+      <c r="M208" s="3" t="n"/>
     </row>
     <row r="209">
       <c r="A209" s="3" t="n"/>
@@ -3119,6 +3773,9 @@
       <c r="H209" s="3" t="n"/>
       <c r="I209" s="3" t="n"/>
       <c r="J209" s="3" t="n"/>
+      <c r="K209" s="3" t="n"/>
+      <c r="L209" s="3" t="n"/>
+      <c r="M209" s="3" t="n"/>
     </row>
     <row r="210">
       <c r="A210" s="3" t="n"/>
@@ -3131,6 +3788,9 @@
       <c r="H210" s="3" t="n"/>
       <c r="I210" s="3" t="n"/>
       <c r="J210" s="3" t="n"/>
+      <c r="K210" s="3" t="n"/>
+      <c r="L210" s="3" t="n"/>
+      <c r="M210" s="3" t="n"/>
     </row>
     <row r="211">
       <c r="A211" s="3" t="n"/>
@@ -3143,6 +3803,9 @@
       <c r="H211" s="3" t="n"/>
       <c r="I211" s="3" t="n"/>
       <c r="J211" s="3" t="n"/>
+      <c r="K211" s="3" t="n"/>
+      <c r="L211" s="3" t="n"/>
+      <c r="M211" s="3" t="n"/>
     </row>
     <row r="212">
       <c r="A212" s="3" t="n"/>
@@ -3155,6 +3818,9 @@
       <c r="H212" s="3" t="n"/>
       <c r="I212" s="3" t="n"/>
       <c r="J212" s="3" t="n"/>
+      <c r="K212" s="3" t="n"/>
+      <c r="L212" s="3" t="n"/>
+      <c r="M212" s="3" t="n"/>
     </row>
     <row r="213">
       <c r="A213" s="3" t="n"/>
@@ -3167,6 +3833,9 @@
       <c r="H213" s="3" t="n"/>
       <c r="I213" s="3" t="n"/>
       <c r="J213" s="3" t="n"/>
+      <c r="K213" s="3" t="n"/>
+      <c r="L213" s="3" t="n"/>
+      <c r="M213" s="3" t="n"/>
     </row>
     <row r="214">
       <c r="A214" s="3" t="n"/>
@@ -3179,6 +3848,9 @@
       <c r="H214" s="3" t="n"/>
       <c r="I214" s="3" t="n"/>
       <c r="J214" s="3" t="n"/>
+      <c r="K214" s="3" t="n"/>
+      <c r="L214" s="3" t="n"/>
+      <c r="M214" s="3" t="n"/>
     </row>
     <row r="215">
       <c r="A215" s="3" t="n"/>
@@ -3191,6 +3863,9 @@
       <c r="H215" s="3" t="n"/>
       <c r="I215" s="3" t="n"/>
       <c r="J215" s="3" t="n"/>
+      <c r="K215" s="3" t="n"/>
+      <c r="L215" s="3" t="n"/>
+      <c r="M215" s="3" t="n"/>
     </row>
     <row r="216">
       <c r="A216" s="3" t="n"/>
@@ -3203,6 +3878,9 @@
       <c r="H216" s="3" t="n"/>
       <c r="I216" s="3" t="n"/>
       <c r="J216" s="3" t="n"/>
+      <c r="K216" s="3" t="n"/>
+      <c r="L216" s="3" t="n"/>
+      <c r="M216" s="3" t="n"/>
     </row>
     <row r="217">
       <c r="A217" s="3" t="n"/>
@@ -3215,6 +3893,9 @@
       <c r="H217" s="3" t="n"/>
       <c r="I217" s="3" t="n"/>
       <c r="J217" s="3" t="n"/>
+      <c r="K217" s="3" t="n"/>
+      <c r="L217" s="3" t="n"/>
+      <c r="M217" s="3" t="n"/>
     </row>
     <row r="218">
       <c r="A218" s="3" t="n"/>
@@ -3227,6 +3908,9 @@
       <c r="H218" s="3" t="n"/>
       <c r="I218" s="3" t="n"/>
       <c r="J218" s="3" t="n"/>
+      <c r="K218" s="3" t="n"/>
+      <c r="L218" s="3" t="n"/>
+      <c r="M218" s="3" t="n"/>
     </row>
     <row r="219">
       <c r="A219" s="3" t="n"/>
@@ -3239,6 +3923,9 @@
       <c r="H219" s="3" t="n"/>
       <c r="I219" s="3" t="n"/>
       <c r="J219" s="3" t="n"/>
+      <c r="K219" s="3" t="n"/>
+      <c r="L219" s="3" t="n"/>
+      <c r="M219" s="3" t="n"/>
     </row>
     <row r="220">
       <c r="A220" s="3" t="n"/>
@@ -3251,6 +3938,9 @@
       <c r="H220" s="3" t="n"/>
       <c r="I220" s="3" t="n"/>
       <c r="J220" s="3" t="n"/>
+      <c r="K220" s="3" t="n"/>
+      <c r="L220" s="3" t="n"/>
+      <c r="M220" s="3" t="n"/>
     </row>
     <row r="221">
       <c r="A221" s="3" t="n"/>
@@ -3263,6 +3953,9 @@
       <c r="H221" s="3" t="n"/>
       <c r="I221" s="3" t="n"/>
       <c r="J221" s="3" t="n"/>
+      <c r="K221" s="3" t="n"/>
+      <c r="L221" s="3" t="n"/>
+      <c r="M221" s="3" t="n"/>
     </row>
     <row r="222">
       <c r="A222" s="3" t="n"/>
@@ -3275,6 +3968,9 @@
       <c r="H222" s="3" t="n"/>
       <c r="I222" s="3" t="n"/>
       <c r="J222" s="3" t="n"/>
+      <c r="K222" s="3" t="n"/>
+      <c r="L222" s="3" t="n"/>
+      <c r="M222" s="3" t="n"/>
     </row>
     <row r="223">
       <c r="A223" s="3" t="n"/>
@@ -3287,6 +3983,9 @@
       <c r="H223" s="3" t="n"/>
       <c r="I223" s="3" t="n"/>
       <c r="J223" s="3" t="n"/>
+      <c r="K223" s="3" t="n"/>
+      <c r="L223" s="3" t="n"/>
+      <c r="M223" s="3" t="n"/>
     </row>
     <row r="224">
       <c r="A224" s="3" t="n"/>
@@ -3299,6 +3998,9 @@
       <c r="H224" s="3" t="n"/>
       <c r="I224" s="3" t="n"/>
       <c r="J224" s="3" t="n"/>
+      <c r="K224" s="3" t="n"/>
+      <c r="L224" s="3" t="n"/>
+      <c r="M224" s="3" t="n"/>
     </row>
     <row r="225">
       <c r="A225" s="3" t="n"/>
@@ -3311,6 +4013,9 @@
       <c r="H225" s="3" t="n"/>
       <c r="I225" s="3" t="n"/>
       <c r="J225" s="3" t="n"/>
+      <c r="K225" s="3" t="n"/>
+      <c r="L225" s="3" t="n"/>
+      <c r="M225" s="3" t="n"/>
     </row>
     <row r="226">
       <c r="A226" s="3" t="n"/>
@@ -3323,6 +4028,9 @@
       <c r="H226" s="3" t="n"/>
       <c r="I226" s="3" t="n"/>
       <c r="J226" s="3" t="n"/>
+      <c r="K226" s="3" t="n"/>
+      <c r="L226" s="3" t="n"/>
+      <c r="M226" s="3" t="n"/>
     </row>
     <row r="227">
       <c r="A227" s="3" t="n"/>
@@ -3335,6 +4043,9 @@
       <c r="H227" s="3" t="n"/>
       <c r="I227" s="3" t="n"/>
       <c r="J227" s="3" t="n"/>
+      <c r="K227" s="3" t="n"/>
+      <c r="L227" s="3" t="n"/>
+      <c r="M227" s="3" t="n"/>
     </row>
     <row r="228">
       <c r="A228" s="3" t="n"/>
@@ -3347,6 +4058,9 @@
       <c r="H228" s="3" t="n"/>
       <c r="I228" s="3" t="n"/>
       <c r="J228" s="3" t="n"/>
+      <c r="K228" s="3" t="n"/>
+      <c r="L228" s="3" t="n"/>
+      <c r="M228" s="3" t="n"/>
     </row>
     <row r="229">
       <c r="A229" s="3" t="n"/>
@@ -3359,6 +4073,9 @@
       <c r="H229" s="3" t="n"/>
       <c r="I229" s="3" t="n"/>
       <c r="J229" s="3" t="n"/>
+      <c r="K229" s="3" t="n"/>
+      <c r="L229" s="3" t="n"/>
+      <c r="M229" s="3" t="n"/>
     </row>
     <row r="230">
       <c r="A230" s="3" t="n"/>
@@ -3371,6 +4088,9 @@
       <c r="H230" s="3" t="n"/>
       <c r="I230" s="3" t="n"/>
       <c r="J230" s="3" t="n"/>
+      <c r="K230" s="3" t="n"/>
+      <c r="L230" s="3" t="n"/>
+      <c r="M230" s="3" t="n"/>
     </row>
     <row r="231">
       <c r="A231" s="3" t="n"/>
@@ -3383,6 +4103,9 @@
       <c r="H231" s="3" t="n"/>
       <c r="I231" s="3" t="n"/>
       <c r="J231" s="3" t="n"/>
+      <c r="K231" s="3" t="n"/>
+      <c r="L231" s="3" t="n"/>
+      <c r="M231" s="3" t="n"/>
     </row>
     <row r="232">
       <c r="A232" s="3" t="n"/>
@@ -3395,6 +4118,9 @@
       <c r="H232" s="3" t="n"/>
       <c r="I232" s="3" t="n"/>
       <c r="J232" s="3" t="n"/>
+      <c r="K232" s="3" t="n"/>
+      <c r="L232" s="3" t="n"/>
+      <c r="M232" s="3" t="n"/>
     </row>
     <row r="233">
       <c r="A233" s="3" t="n"/>
@@ -3407,6 +4133,9 @@
       <c r="H233" s="3" t="n"/>
       <c r="I233" s="3" t="n"/>
       <c r="J233" s="3" t="n"/>
+      <c r="K233" s="3" t="n"/>
+      <c r="L233" s="3" t="n"/>
+      <c r="M233" s="3" t="n"/>
     </row>
     <row r="234">
       <c r="A234" s="3" t="n"/>
@@ -3419,6 +4148,9 @@
       <c r="H234" s="3" t="n"/>
       <c r="I234" s="3" t="n"/>
       <c r="J234" s="3" t="n"/>
+      <c r="K234" s="3" t="n"/>
+      <c r="L234" s="3" t="n"/>
+      <c r="M234" s="3" t="n"/>
     </row>
     <row r="235">
       <c r="A235" s="3" t="n"/>
@@ -3431,6 +4163,9 @@
       <c r="H235" s="3" t="n"/>
       <c r="I235" s="3" t="n"/>
       <c r="J235" s="3" t="n"/>
+      <c r="K235" s="3" t="n"/>
+      <c r="L235" s="3" t="n"/>
+      <c r="M235" s="3" t="n"/>
     </row>
     <row r="236">
       <c r="A236" s="3" t="n"/>
@@ -3443,6 +4178,9 @@
       <c r="H236" s="3" t="n"/>
       <c r="I236" s="3" t="n"/>
       <c r="J236" s="3" t="n"/>
+      <c r="K236" s="3" t="n"/>
+      <c r="L236" s="3" t="n"/>
+      <c r="M236" s="3" t="n"/>
     </row>
     <row r="237">
       <c r="A237" s="3" t="n"/>
@@ -3455,6 +4193,9 @@
       <c r="H237" s="3" t="n"/>
       <c r="I237" s="3" t="n"/>
       <c r="J237" s="3" t="n"/>
+      <c r="K237" s="3" t="n"/>
+      <c r="L237" s="3" t="n"/>
+      <c r="M237" s="3" t="n"/>
     </row>
     <row r="238">
       <c r="A238" s="3" t="n"/>
@@ -3467,6 +4208,9 @@
       <c r="H238" s="3" t="n"/>
       <c r="I238" s="3" t="n"/>
       <c r="J238" s="3" t="n"/>
+      <c r="K238" s="3" t="n"/>
+      <c r="L238" s="3" t="n"/>
+      <c r="M238" s="3" t="n"/>
     </row>
     <row r="239">
       <c r="A239" s="3" t="n"/>
@@ -3479,6 +4223,9 @@
       <c r="H239" s="3" t="n"/>
       <c r="I239" s="3" t="n"/>
       <c r="J239" s="3" t="n"/>
+      <c r="K239" s="3" t="n"/>
+      <c r="L239" s="3" t="n"/>
+      <c r="M239" s="3" t="n"/>
     </row>
     <row r="240">
       <c r="A240" s="3" t="n"/>
@@ -3491,6 +4238,9 @@
       <c r="H240" s="3" t="n"/>
       <c r="I240" s="3" t="n"/>
       <c r="J240" s="3" t="n"/>
+      <c r="K240" s="3" t="n"/>
+      <c r="L240" s="3" t="n"/>
+      <c r="M240" s="3" t="n"/>
     </row>
     <row r="241">
       <c r="A241" s="3" t="n"/>
@@ -3503,6 +4253,9 @@
       <c r="H241" s="3" t="n"/>
       <c r="I241" s="3" t="n"/>
       <c r="J241" s="3" t="n"/>
+      <c r="K241" s="3" t="n"/>
+      <c r="L241" s="3" t="n"/>
+      <c r="M241" s="3" t="n"/>
     </row>
     <row r="242">
       <c r="A242" s="3" t="n"/>
@@ -3515,6 +4268,9 @@
       <c r="H242" s="3" t="n"/>
       <c r="I242" s="3" t="n"/>
       <c r="J242" s="3" t="n"/>
+      <c r="K242" s="3" t="n"/>
+      <c r="L242" s="3" t="n"/>
+      <c r="M242" s="3" t="n"/>
     </row>
     <row r="243">
       <c r="A243" s="3" t="n"/>
@@ -3527,6 +4283,9 @@
       <c r="H243" s="3" t="n"/>
       <c r="I243" s="3" t="n"/>
       <c r="J243" s="3" t="n"/>
+      <c r="K243" s="3" t="n"/>
+      <c r="L243" s="3" t="n"/>
+      <c r="M243" s="3" t="n"/>
     </row>
     <row r="244">
       <c r="A244" s="3" t="n"/>
@@ -3539,6 +4298,9 @@
       <c r="H244" s="3" t="n"/>
       <c r="I244" s="3" t="n"/>
       <c r="J244" s="3" t="n"/>
+      <c r="K244" s="3" t="n"/>
+      <c r="L244" s="3" t="n"/>
+      <c r="M244" s="3" t="n"/>
     </row>
     <row r="245">
       <c r="A245" s="3" t="n"/>
@@ -3551,6 +4313,9 @@
       <c r="H245" s="3" t="n"/>
       <c r="I245" s="3" t="n"/>
       <c r="J245" s="3" t="n"/>
+      <c r="K245" s="3" t="n"/>
+      <c r="L245" s="3" t="n"/>
+      <c r="M245" s="3" t="n"/>
     </row>
     <row r="246">
       <c r="A246" s="3" t="n"/>
@@ -3563,6 +4328,9 @@
       <c r="H246" s="3" t="n"/>
       <c r="I246" s="3" t="n"/>
       <c r="J246" s="3" t="n"/>
+      <c r="K246" s="3" t="n"/>
+      <c r="L246" s="3" t="n"/>
+      <c r="M246" s="3" t="n"/>
     </row>
     <row r="247">
       <c r="A247" s="3" t="n"/>
@@ -3575,6 +4343,9 @@
       <c r="H247" s="3" t="n"/>
       <c r="I247" s="3" t="n"/>
       <c r="J247" s="3" t="n"/>
+      <c r="K247" s="3" t="n"/>
+      <c r="L247" s="3" t="n"/>
+      <c r="M247" s="3" t="n"/>
     </row>
     <row r="248">
       <c r="A248" s="3" t="n"/>
@@ -3587,6 +4358,9 @@
       <c r="H248" s="3" t="n"/>
       <c r="I248" s="3" t="n"/>
       <c r="J248" s="3" t="n"/>
+      <c r="K248" s="3" t="n"/>
+      <c r="L248" s="3" t="n"/>
+      <c r="M248" s="3" t="n"/>
     </row>
     <row r="249">
       <c r="A249" s="3" t="n"/>
@@ -3599,6 +4373,9 @@
       <c r="H249" s="3" t="n"/>
       <c r="I249" s="3" t="n"/>
       <c r="J249" s="3" t="n"/>
+      <c r="K249" s="3" t="n"/>
+      <c r="L249" s="3" t="n"/>
+      <c r="M249" s="3" t="n"/>
     </row>
     <row r="250">
       <c r="A250" s="3" t="n"/>
@@ -3611,6 +4388,9 @@
       <c r="H250" s="3" t="n"/>
       <c r="I250" s="3" t="n"/>
       <c r="J250" s="3" t="n"/>
+      <c r="K250" s="3" t="n"/>
+      <c r="L250" s="3" t="n"/>
+      <c r="M250" s="3" t="n"/>
     </row>
     <row r="251">
       <c r="A251" s="3" t="n"/>
@@ -3623,6 +4403,9 @@
       <c r="H251" s="3" t="n"/>
       <c r="I251" s="3" t="n"/>
       <c r="J251" s="3" t="n"/>
+      <c r="K251" s="3" t="n"/>
+      <c r="L251" s="3" t="n"/>
+      <c r="M251" s="3" t="n"/>
     </row>
     <row r="252">
       <c r="A252" s="3" t="n"/>
@@ -3635,6 +4418,9 @@
       <c r="H252" s="3" t="n"/>
       <c r="I252" s="3" t="n"/>
       <c r="J252" s="3" t="n"/>
+      <c r="K252" s="3" t="n"/>
+      <c r="L252" s="3" t="n"/>
+      <c r="M252" s="3" t="n"/>
     </row>
     <row r="253">
       <c r="A253" s="3" t="n"/>
@@ -3647,6 +4433,9 @@
       <c r="H253" s="3" t="n"/>
       <c r="I253" s="3" t="n"/>
       <c r="J253" s="3" t="n"/>
+      <c r="K253" s="3" t="n"/>
+      <c r="L253" s="3" t="n"/>
+      <c r="M253" s="3" t="n"/>
     </row>
     <row r="254">
       <c r="A254" s="3" t="n"/>
@@ -3659,6 +4448,9 @@
       <c r="H254" s="3" t="n"/>
       <c r="I254" s="3" t="n"/>
       <c r="J254" s="3" t="n"/>
+      <c r="K254" s="3" t="n"/>
+      <c r="L254" s="3" t="n"/>
+      <c r="M254" s="3" t="n"/>
     </row>
     <row r="255">
       <c r="A255" s="3" t="n"/>
@@ -3671,6 +4463,9 @@
       <c r="H255" s="3" t="n"/>
       <c r="I255" s="3" t="n"/>
       <c r="J255" s="3" t="n"/>
+      <c r="K255" s="3" t="n"/>
+      <c r="L255" s="3" t="n"/>
+      <c r="M255" s="3" t="n"/>
     </row>
     <row r="256">
       <c r="A256" s="3" t="n"/>
@@ -3683,6 +4478,9 @@
       <c r="H256" s="3" t="n"/>
       <c r="I256" s="3" t="n"/>
       <c r="J256" s="3" t="n"/>
+      <c r="K256" s="3" t="n"/>
+      <c r="L256" s="3" t="n"/>
+      <c r="M256" s="3" t="n"/>
     </row>
     <row r="257">
       <c r="A257" s="3" t="n"/>
@@ -3695,6 +4493,9 @@
       <c r="H257" s="3" t="n"/>
       <c r="I257" s="3" t="n"/>
       <c r="J257" s="3" t="n"/>
+      <c r="K257" s="3" t="n"/>
+      <c r="L257" s="3" t="n"/>
+      <c r="M257" s="3" t="n"/>
     </row>
     <row r="258">
       <c r="A258" s="3" t="n"/>
@@ -3707,6 +4508,9 @@
       <c r="H258" s="3" t="n"/>
       <c r="I258" s="3" t="n"/>
       <c r="J258" s="3" t="n"/>
+      <c r="K258" s="3" t="n"/>
+      <c r="L258" s="3" t="n"/>
+      <c r="M258" s="3" t="n"/>
     </row>
     <row r="259">
       <c r="A259" s="3" t="n"/>
@@ -3719,6 +4523,9 @@
       <c r="H259" s="3" t="n"/>
       <c r="I259" s="3" t="n"/>
       <c r="J259" s="3" t="n"/>
+      <c r="K259" s="3" t="n"/>
+      <c r="L259" s="3" t="n"/>
+      <c r="M259" s="3" t="n"/>
     </row>
     <row r="260">
       <c r="A260" s="3" t="n"/>
@@ -3731,6 +4538,9 @@
       <c r="H260" s="3" t="n"/>
       <c r="I260" s="3" t="n"/>
       <c r="J260" s="3" t="n"/>
+      <c r="K260" s="3" t="n"/>
+      <c r="L260" s="3" t="n"/>
+      <c r="M260" s="3" t="n"/>
     </row>
     <row r="261">
       <c r="A261" s="3" t="n"/>
@@ -3743,6 +4553,9 @@
       <c r="H261" s="3" t="n"/>
       <c r="I261" s="3" t="n"/>
       <c r="J261" s="3" t="n"/>
+      <c r="K261" s="3" t="n"/>
+      <c r="L261" s="3" t="n"/>
+      <c r="M261" s="3" t="n"/>
     </row>
     <row r="262">
       <c r="A262" s="3" t="n"/>
@@ -3755,6 +4568,9 @@
       <c r="H262" s="3" t="n"/>
       <c r="I262" s="3" t="n"/>
       <c r="J262" s="3" t="n"/>
+      <c r="K262" s="3" t="n"/>
+      <c r="L262" s="3" t="n"/>
+      <c r="M262" s="3" t="n"/>
     </row>
     <row r="263">
       <c r="A263" s="3" t="n"/>
@@ -3767,6 +4583,9 @@
       <c r="H263" s="3" t="n"/>
       <c r="I263" s="3" t="n"/>
       <c r="J263" s="3" t="n"/>
+      <c r="K263" s="3" t="n"/>
+      <c r="L263" s="3" t="n"/>
+      <c r="M263" s="3" t="n"/>
     </row>
     <row r="264">
       <c r="A264" s="3" t="n"/>
@@ -3779,6 +4598,9 @@
       <c r="H264" s="3" t="n"/>
       <c r="I264" s="3" t="n"/>
       <c r="J264" s="3" t="n"/>
+      <c r="K264" s="3" t="n"/>
+      <c r="L264" s="3" t="n"/>
+      <c r="M264" s="3" t="n"/>
     </row>
     <row r="265">
       <c r="A265" s="3" t="n"/>
@@ -3791,6 +4613,9 @@
       <c r="H265" s="3" t="n"/>
       <c r="I265" s="3" t="n"/>
       <c r="J265" s="3" t="n"/>
+      <c r="K265" s="3" t="n"/>
+      <c r="L265" s="3" t="n"/>
+      <c r="M265" s="3" t="n"/>
     </row>
     <row r="266">
       <c r="A266" s="3" t="n"/>
@@ -3803,6 +4628,9 @@
       <c r="H266" s="3" t="n"/>
       <c r="I266" s="3" t="n"/>
       <c r="J266" s="3" t="n"/>
+      <c r="K266" s="3" t="n"/>
+      <c r="L266" s="3" t="n"/>
+      <c r="M266" s="3" t="n"/>
     </row>
     <row r="267">
       <c r="A267" s="3" t="n"/>
@@ -3815,6 +4643,9 @@
       <c r="H267" s="3" t="n"/>
       <c r="I267" s="3" t="n"/>
       <c r="J267" s="3" t="n"/>
+      <c r="K267" s="3" t="n"/>
+      <c r="L267" s="3" t="n"/>
+      <c r="M267" s="3" t="n"/>
     </row>
     <row r="268">
       <c r="A268" s="3" t="n"/>
@@ -3827,6 +4658,9 @@
       <c r="H268" s="3" t="n"/>
       <c r="I268" s="3" t="n"/>
       <c r="J268" s="3" t="n"/>
+      <c r="K268" s="3" t="n"/>
+      <c r="L268" s="3" t="n"/>
+      <c r="M268" s="3" t="n"/>
     </row>
     <row r="269">
       <c r="A269" s="3" t="n"/>
@@ -3839,6 +4673,9 @@
       <c r="H269" s="3" t="n"/>
       <c r="I269" s="3" t="n"/>
       <c r="J269" s="3" t="n"/>
+      <c r="K269" s="3" t="n"/>
+      <c r="L269" s="3" t="n"/>
+      <c r="M269" s="3" t="n"/>
     </row>
     <row r="270">
       <c r="A270" s="3" t="n"/>
@@ -3851,6 +4688,9 @@
       <c r="H270" s="3" t="n"/>
       <c r="I270" s="3" t="n"/>
       <c r="J270" s="3" t="n"/>
+      <c r="K270" s="3" t="n"/>
+      <c r="L270" s="3" t="n"/>
+      <c r="M270" s="3" t="n"/>
     </row>
     <row r="271">
       <c r="A271" s="3" t="n"/>
@@ -3863,6 +4703,9 @@
       <c r="H271" s="3" t="n"/>
       <c r="I271" s="3" t="n"/>
       <c r="J271" s="3" t="n"/>
+      <c r="K271" s="3" t="n"/>
+      <c r="L271" s="3" t="n"/>
+      <c r="M271" s="3" t="n"/>
     </row>
     <row r="272">
       <c r="A272" s="3" t="n"/>
@@ -3875,6 +4718,9 @@
       <c r="H272" s="3" t="n"/>
       <c r="I272" s="3" t="n"/>
       <c r="J272" s="3" t="n"/>
+      <c r="K272" s="3" t="n"/>
+      <c r="L272" s="3" t="n"/>
+      <c r="M272" s="3" t="n"/>
     </row>
     <row r="273">
       <c r="A273" s="3" t="n"/>
@@ -3887,6 +4733,9 @@
       <c r="H273" s="3" t="n"/>
       <c r="I273" s="3" t="n"/>
       <c r="J273" s="3" t="n"/>
+      <c r="K273" s="3" t="n"/>
+      <c r="L273" s="3" t="n"/>
+      <c r="M273" s="3" t="n"/>
     </row>
     <row r="274">
       <c r="A274" s="3" t="n"/>
@@ -3899,6 +4748,9 @@
       <c r="H274" s="3" t="n"/>
       <c r="I274" s="3" t="n"/>
       <c r="J274" s="3" t="n"/>
+      <c r="K274" s="3" t="n"/>
+      <c r="L274" s="3" t="n"/>
+      <c r="M274" s="3" t="n"/>
     </row>
     <row r="275">
       <c r="A275" s="3" t="n"/>
@@ -3911,6 +4763,9 @@
       <c r="H275" s="3" t="n"/>
       <c r="I275" s="3" t="n"/>
       <c r="J275" s="3" t="n"/>
+      <c r="K275" s="3" t="n"/>
+      <c r="L275" s="3" t="n"/>
+      <c r="M275" s="3" t="n"/>
     </row>
     <row r="276">
       <c r="A276" s="3" t="n"/>
@@ -3923,6 +4778,9 @@
       <c r="H276" s="3" t="n"/>
       <c r="I276" s="3" t="n"/>
       <c r="J276" s="3" t="n"/>
+      <c r="K276" s="3" t="n"/>
+      <c r="L276" s="3" t="n"/>
+      <c r="M276" s="3" t="n"/>
     </row>
     <row r="277">
       <c r="A277" s="3" t="n"/>
@@ -3935,6 +4793,9 @@
       <c r="H277" s="3" t="n"/>
       <c r="I277" s="3" t="n"/>
       <c r="J277" s="3" t="n"/>
+      <c r="K277" s="3" t="n"/>
+      <c r="L277" s="3" t="n"/>
+      <c r="M277" s="3" t="n"/>
     </row>
     <row r="278">
       <c r="A278" s="3" t="n"/>
@@ -3947,6 +4808,9 @@
       <c r="H278" s="3" t="n"/>
       <c r="I278" s="3" t="n"/>
       <c r="J278" s="3" t="n"/>
+      <c r="K278" s="3" t="n"/>
+      <c r="L278" s="3" t="n"/>
+      <c r="M278" s="3" t="n"/>
     </row>
     <row r="279">
       <c r="A279" s="3" t="n"/>
@@ -3959,6 +4823,9 @@
       <c r="H279" s="3" t="n"/>
       <c r="I279" s="3" t="n"/>
       <c r="J279" s="3" t="n"/>
+      <c r="K279" s="3" t="n"/>
+      <c r="L279" s="3" t="n"/>
+      <c r="M279" s="3" t="n"/>
     </row>
     <row r="280">
       <c r="A280" s="3" t="n"/>
@@ -3971,6 +4838,9 @@
       <c r="H280" s="3" t="n"/>
       <c r="I280" s="3" t="n"/>
       <c r="J280" s="3" t="n"/>
+      <c r="K280" s="3" t="n"/>
+      <c r="L280" s="3" t="n"/>
+      <c r="M280" s="3" t="n"/>
     </row>
     <row r="281">
       <c r="A281" s="3" t="n"/>
@@ -3983,6 +4853,9 @@
       <c r="H281" s="3" t="n"/>
       <c r="I281" s="3" t="n"/>
       <c r="J281" s="3" t="n"/>
+      <c r="K281" s="3" t="n"/>
+      <c r="L281" s="3" t="n"/>
+      <c r="M281" s="3" t="n"/>
     </row>
     <row r="282">
       <c r="A282" s="3" t="n"/>
@@ -3995,6 +4868,9 @@
       <c r="H282" s="3" t="n"/>
       <c r="I282" s="3" t="n"/>
       <c r="J282" s="3" t="n"/>
+      <c r="K282" s="3" t="n"/>
+      <c r="L282" s="3" t="n"/>
+      <c r="M282" s="3" t="n"/>
     </row>
     <row r="283">
       <c r="A283" s="3" t="n"/>
@@ -4007,6 +4883,9 @@
       <c r="H283" s="3" t="n"/>
       <c r="I283" s="3" t="n"/>
       <c r="J283" s="3" t="n"/>
+      <c r="K283" s="3" t="n"/>
+      <c r="L283" s="3" t="n"/>
+      <c r="M283" s="3" t="n"/>
     </row>
     <row r="284">
       <c r="A284" s="3" t="n"/>
@@ -4019,6 +4898,9 @@
       <c r="H284" s="3" t="n"/>
       <c r="I284" s="3" t="n"/>
       <c r="J284" s="3" t="n"/>
+      <c r="K284" s="3" t="n"/>
+      <c r="L284" s="3" t="n"/>
+      <c r="M284" s="3" t="n"/>
     </row>
     <row r="285">
       <c r="A285" s="3" t="n"/>
@@ -4031,6 +4913,9 @@
       <c r="H285" s="3" t="n"/>
       <c r="I285" s="3" t="n"/>
       <c r="J285" s="3" t="n"/>
+      <c r="K285" s="3" t="n"/>
+      <c r="L285" s="3" t="n"/>
+      <c r="M285" s="3" t="n"/>
     </row>
     <row r="286">
       <c r="A286" s="3" t="n"/>
@@ -4043,6 +4928,9 @@
       <c r="H286" s="3" t="n"/>
       <c r="I286" s="3" t="n"/>
       <c r="J286" s="3" t="n"/>
+      <c r="K286" s="3" t="n"/>
+      <c r="L286" s="3" t="n"/>
+      <c r="M286" s="3" t="n"/>
     </row>
     <row r="287">
       <c r="A287" s="3" t="n"/>
@@ -4055,6 +4943,9 @@
       <c r="H287" s="3" t="n"/>
       <c r="I287" s="3" t="n"/>
       <c r="J287" s="3" t="n"/>
+      <c r="K287" s="3" t="n"/>
+      <c r="L287" s="3" t="n"/>
+      <c r="M287" s="3" t="n"/>
     </row>
     <row r="288">
       <c r="A288" s="3" t="n"/>
@@ -4067,6 +4958,9 @@
       <c r="H288" s="3" t="n"/>
       <c r="I288" s="3" t="n"/>
       <c r="J288" s="3" t="n"/>
+      <c r="K288" s="3" t="n"/>
+      <c r="L288" s="3" t="n"/>
+      <c r="M288" s="3" t="n"/>
     </row>
     <row r="289">
       <c r="A289" s="3" t="n"/>
@@ -4079,6 +4973,9 @@
       <c r="H289" s="3" t="n"/>
       <c r="I289" s="3" t="n"/>
       <c r="J289" s="3" t="n"/>
+      <c r="K289" s="3" t="n"/>
+      <c r="L289" s="3" t="n"/>
+      <c r="M289" s="3" t="n"/>
     </row>
     <row r="290">
       <c r="A290" s="3" t="n"/>
@@ -4091,6 +4988,9 @@
       <c r="H290" s="3" t="n"/>
       <c r="I290" s="3" t="n"/>
       <c r="J290" s="3" t="n"/>
+      <c r="K290" s="3" t="n"/>
+      <c r="L290" s="3" t="n"/>
+      <c r="M290" s="3" t="n"/>
     </row>
     <row r="291">
       <c r="A291" s="3" t="n"/>
@@ -4103,6 +5003,9 @@
       <c r="H291" s="3" t="n"/>
       <c r="I291" s="3" t="n"/>
       <c r="J291" s="3" t="n"/>
+      <c r="K291" s="3" t="n"/>
+      <c r="L291" s="3" t="n"/>
+      <c r="M291" s="3" t="n"/>
     </row>
     <row r="292">
       <c r="A292" s="3" t="n"/>
@@ -4115,6 +5018,9 @@
       <c r="H292" s="3" t="n"/>
       <c r="I292" s="3" t="n"/>
       <c r="J292" s="3" t="n"/>
+      <c r="K292" s="3" t="n"/>
+      <c r="L292" s="3" t="n"/>
+      <c r="M292" s="3" t="n"/>
     </row>
     <row r="293">
       <c r="A293" s="3" t="n"/>
@@ -4127,6 +5033,9 @@
       <c r="H293" s="3" t="n"/>
       <c r="I293" s="3" t="n"/>
       <c r="J293" s="3" t="n"/>
+      <c r="K293" s="3" t="n"/>
+      <c r="L293" s="3" t="n"/>
+      <c r="M293" s="3" t="n"/>
     </row>
     <row r="294">
       <c r="A294" s="3" t="n"/>
@@ -4139,6 +5048,9 @@
       <c r="H294" s="3" t="n"/>
       <c r="I294" s="3" t="n"/>
       <c r="J294" s="3" t="n"/>
+      <c r="K294" s="3" t="n"/>
+      <c r="L294" s="3" t="n"/>
+      <c r="M294" s="3" t="n"/>
     </row>
     <row r="295">
       <c r="A295" s="3" t="n"/>
@@ -4151,6 +5063,9 @@
       <c r="H295" s="3" t="n"/>
       <c r="I295" s="3" t="n"/>
       <c r="J295" s="3" t="n"/>
+      <c r="K295" s="3" t="n"/>
+      <c r="L295" s="3" t="n"/>
+      <c r="M295" s="3" t="n"/>
     </row>
     <row r="296">
       <c r="A296" s="3" t="n"/>
@@ -4163,6 +5078,9 @@
       <c r="H296" s="3" t="n"/>
       <c r="I296" s="3" t="n"/>
       <c r="J296" s="3" t="n"/>
+      <c r="K296" s="3" t="n"/>
+      <c r="L296" s="3" t="n"/>
+      <c r="M296" s="3" t="n"/>
     </row>
     <row r="297">
       <c r="A297" s="3" t="n"/>
@@ -4175,6 +5093,9 @@
       <c r="H297" s="3" t="n"/>
       <c r="I297" s="3" t="n"/>
       <c r="J297" s="3" t="n"/>
+      <c r="K297" s="3" t="n"/>
+      <c r="L297" s="3" t="n"/>
+      <c r="M297" s="3" t="n"/>
     </row>
     <row r="298">
       <c r="A298" s="3" t="n"/>
@@ -4187,6 +5108,9 @@
       <c r="H298" s="3" t="n"/>
       <c r="I298" s="3" t="n"/>
       <c r="J298" s="3" t="n"/>
+      <c r="K298" s="3" t="n"/>
+      <c r="L298" s="3" t="n"/>
+      <c r="M298" s="3" t="n"/>
     </row>
     <row r="299">
       <c r="A299" s="3" t="n"/>
@@ -4199,6 +5123,9 @@
       <c r="H299" s="3" t="n"/>
       <c r="I299" s="3" t="n"/>
       <c r="J299" s="3" t="n"/>
+      <c r="K299" s="3" t="n"/>
+      <c r="L299" s="3" t="n"/>
+      <c r="M299" s="3" t="n"/>
     </row>
     <row r="300">
       <c r="A300" s="3" t="n"/>
@@ -4211,6 +5138,9 @@
       <c r="H300" s="3" t="n"/>
       <c r="I300" s="3" t="n"/>
       <c r="J300" s="3" t="n"/>
+      <c r="K300" s="3" t="n"/>
+      <c r="L300" s="3" t="n"/>
+      <c r="M300" s="3" t="n"/>
     </row>
     <row r="301">
       <c r="A301" s="3" t="n"/>
@@ -4223,9 +5153,12 @@
       <c r="H301" s="3" t="n"/>
       <c r="I301" s="3" t="n"/>
       <c r="J301" s="3" t="n"/>
+      <c r="K301" s="3" t="n"/>
+      <c r="L301" s="3" t="n"/>
+      <c r="M301" s="3" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="7">
+  <dataValidations count="10">
     <dataValidation sqref="F2:F301" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Papel" error="Use instrutor ou aluno." type="list" errorStyle="stop">
       <formula1>"instrutor,aluno"</formula1>
     </dataValidation>
@@ -4246,6 +5179,18 @@
       <formula1>6</formula1>
       <formula2>72</formula2>
     </dataValidation>
+    <dataValidation sqref="K2:K301" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Número à esquerda" error="De 1 a 4 caracteres (ou deixe vazio)." type="textLength" errorStyle="stop" operator="between">
+      <formula1>1</formula1>
+      <formula2>4</formula2>
+    </dataValidation>
+    <dataValidation sqref="L2:L301" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Número à direita" error="De 1 a 4 caracteres (ou deixe vazio)." type="textLength" errorStyle="stop" operator="between">
+      <formula1>1</formula1>
+      <formula2>4</formula2>
+    </dataValidation>
+    <dataValidation sqref="M2:M301" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nome da fração" error="De 1 a 20 caracteres (ou deixe vazio)." type="textLength" errorStyle="stop" operator="between">
+      <formula1>1</formula1>
+      <formula2>20</formula2>
+    </dataValidation>
     <dataValidation sqref="D2:D301" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nome de guerra" error="De 1 a 30 caracteres." type="textLength" errorStyle="stop" operator="between">
       <formula1>1</formula1>
       <formula2>30</formula2>
@@ -4262,7 +5207,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:B21"/>
+  <dimension ref="B1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -4377,21 +5322,35 @@
     <row r="18" ht="32" customHeight="1">
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>• Nome de guerra: é o que aparece no mapa. Curto (até 30 caracteres).</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="B20" s="5" t="inlineStr">
+          <t>• Nome de guerra: até 30 caracteres. Aparece ao lado do símbolo no mapa só quando a pessoa NÃO tem número à esquerda nem à direita.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="32" customHeight="1">
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>• Designação do símbolo (colunas numero_esq e numero_dir): o número da ESQUERDA diz qual é a fração e o da DIREITA diz de quem ela é. Ex.: o 1º Pelotão do 2º Esquadrão é esq = 1, dir = 2, com escalão PEL — os três pontos em cima do símbolo vêm do escalão. Até 4 caracteres cada. Com pelo menos um número preenchido, o nome de guerra deixa de aparecer no desenho (você reconhece a conta pelo usuário). Vazio nos dois = como antes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="32" customHeight="1">
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>• Nome da fração (coluna nome_fracao): texto livre, até 20 caracteres. Aparece só no popup, ao clicar no símbolo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>Exemplo (aba "Exemplo")</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="30" customHeight="1">
-      <c r="B21" s="6" t="inlineStr">
-        <is>
-          <t>A aba "Exemplo" mostra três linhas realistas. Ela NÃO é lida na importação (só a primeira aba é exportada como CSV); não apague nem preencha nela.</t>
+    <row r="23" ht="30" customHeight="1">
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>A aba "Exemplo" mostra três linhas realistas (o aluno01 é o 1º Pelotão do 2º Esqd: 1 [símbolo] 2). Ela NÃO é lida na importação (só a primeira aba é exportada como CSV); não apague nem preencha nela.</t>
         </is>
       </c>
     </row>
@@ -4732,7 +5691,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4745,6 +5704,9 @@
     <col width="28" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4798,6 +5760,21 @@
           <t>natureza_code</t>
         </is>
       </c>
+      <c r="K1" s="10" t="inlineStr">
+        <is>
+          <t>numero_esq</t>
+        </is>
+      </c>
+      <c r="L1" s="10" t="inlineStr">
+        <is>
+          <t>numero_dir</t>
+        </is>
+      </c>
+      <c r="M1" s="10" t="inlineStr">
+        <is>
+          <t>nome_fracao</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
@@ -4842,6 +5819,9 @@
         </is>
       </c>
       <c r="J2" s="11" t="inlineStr"/>
+      <c r="K2" s="11" t="inlineStr"/>
+      <c r="L2" s="11" t="inlineStr"/>
+      <c r="M2" s="11" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="11" t="inlineStr">
@@ -4890,6 +5870,21 @@
         </is>
       </c>
       <c r="J3" s="11" t="inlineStr"/>
+      <c r="K3" s="11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L3" s="11" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="M3" s="11" t="inlineStr">
+        <is>
+          <t>1º Pel / 2º Esqd</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
@@ -4934,11 +5929,27 @@
       </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
-          <t>SEC</t>
+          <t>PEL</t>
         </is>
       </c>
       <c r="J4" s="11" t="inlineStr"/>
-    </row>
+      <c r="K4" s="11" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L4" s="11" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="M4" s="11" t="inlineStr">
+        <is>
+          <t>2º Pel / 2º Esqd</t>
+        </is>
+      </c>
+    </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
         <is>

</xml_diff>